<commit_message>
Complete phase 2 Fabric identity enforcement
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rfa0ab86c47c14e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R92332589e1f94ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R6afd6e98fd774d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rad0d887e9c0742ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R8803d432a99f49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R08582bdcf87d4861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6a6cecd44f2c4dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="Rd434e3b4453b4baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="Rd9dfc3edc49a4c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rff780bfacbd24074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R53f729e8ab194b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="Rd9185245136849c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R6bf5b8ad980f43d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1351,9 +1352,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Chaincode RBAC</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Existing RBAC checks remain commented out. This should be addressed as a security/design decision rather than silently changed.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Mobile app runtime</x:t>
@@ -1469,7 +1467,7 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1546,6 +1544,16 @@
         <x:fgColor rgb="FF000000"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F3A5F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF000000"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -1593,7 +1601,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1692,6 +1700,19 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2383,7 +2404,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33884aa885264c3a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R88eeefad4fa7410e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2393,8 +2414,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangesTable" displayName="ChangesTable" ref="A1:G83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="34" headerRowBorderDxfId="32">
-  <x:autoFilter ref="A1:G83"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangesTable" displayName="ChangesTable" ref="A1:G87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="34" headerRowBorderDxfId="32">
+  <x:autoFilter ref="A1:G87"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Category"/>
@@ -2423,8 +2444,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VerificationTable" displayName="VerificationTable" ref="A1:C19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="9">
-  <x:autoFilter ref="A1:C19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VerificationTable" displayName="VerificationTable" ref="A1:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="9">
+  <x:autoFilter ref="A1:C25"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Verification Item"/>
     <x:tableColumn id="2" name="Result"/>
@@ -2435,8 +2456,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="KnownItemsTable" displayName="KnownItemsTable" ref="A1:B9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="1">
-  <x:autoFilter ref="A1:B9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="KnownItemsTable" displayName="KnownItemsTable" ref="A1:B10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="1">
+  <x:autoFilter ref="A1:B10"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Status / Note"/>
@@ -2800,7 +2821,7 @@
     <x:mergeCell ref="A8:H8"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84df101d7c884be8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cc5b93e43b14815"/>
 </x:worksheet>
 </file>
 
@@ -4723,6 +4744,98 @@
       </x:c>
       <x:c r="G83" t="str">
         <x:v>Gives every future thread a concrete migration and smoke-test checklist before moving to Phase 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>P2-04</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>Tests / Deployment</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>chaincode tests; dental-backend tests; AWS Fabric basic 1.0.1 sequence 3</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>Phase 2 verification</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>No deployed evidence tied role-bound certificates to live chaincode enforcement.</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>Added 16 unit tests, 4 JWT-to-wallet resolver tests, 9 live gateway identity checks, and deployed chaincode sequence 3 with both MSP approvals.</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>Provides repeatable Phase 2 security evidence and confirms deployment behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>P2-03</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>Fabric Identity</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>dental-backend/registerRoleIdentities.js; dental-backend/.env.example</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>role identity enrollment</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>The wallet contained only admin and shared appUser identities.</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>Provisions clinic-bound admin, actor-bound doctor/patient, and system X.509 identities with ecert attributes.</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Makes chaincode role, actor, and clinic checks available from certificate claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>P2-02</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>dental-backend/index.js; dental-backend/fabricIdentity.js</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>gateway identity selection</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Fabric gateway transactions assumed a shared appUser identity.</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>Maps verified JWT context to admin-, doctor-, patient-, or system wallet labels and rejects missing identities before connection.</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>Prevents API users from sharing one Fabric transaction identity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>P2-01</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Fabric / Chaincode</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>fabric-samples/dental-record-sharing/chaincode-javascript/lib/dentalRecordSharing.js; test/dentallRecordSharing_test.js</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>31-66; Phase 2 identity tests</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Chaincode role checks did not reject an invoking certificate from an untrusted MSP.</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Added _requireMsp validation for Org1MSP/Org2MSP before role checks and added an unknown-MSP role-violation test.</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>Starts Phase 2 SEC-02 MSP enforcement after the AWS Phase 1 deployment gate passed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4748,7 +4861,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1633f2bb6c9b489d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac9f42c19ee8484a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4919,7 +5032,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43751d10f70c44ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5debd18d7094971"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5059,7 +5172,7 @@
       <x:c r="B11" t="str">
         <x:v>Pass. node --check succeeded for backend/server.js and dental-backend/index.js.</x:v>
       </x:c>
-      <x:c r="C11" s="48" t="str">
+      <x:c r="C11" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5070,7 +5183,7 @@
       <x:c r="B12" t="str">
         <x:v>Pass. package.json and package-lock.json parse after adding jsonwebtoken.</x:v>
       </x:c>
-      <x:c r="C12" s="48" t="str">
+      <x:c r="C12" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5081,7 +5194,7 @@
       <x:c r="B13" t="str">
         <x:v>Pass. No active Patient1/API_BASE_URL protected request calls found.</x:v>
       </x:c>
-      <x:c r="C13" s="48" t="str">
+      <x:c r="C13" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5092,7 +5205,7 @@
       <x:c r="B14" t="str">
         <x:v>Pass. node --check succeeded for backend/server.js, dental-backend/index.js, and BC-Dentistry-Mobile-App/utils/api.js.</x:v>
       </x:c>
-      <x:c r="C14" s="48" t="str">
+      <x:c r="C14" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5103,7 +5216,7 @@
       <x:c r="B15" t="str">
         <x:v>Pass. requirePatientSelfParam/body middleware is applied to patient request and consent routes.</x:v>
       </x:c>
-      <x:c r="C15" s="48" t="str">
+      <x:c r="C15" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5114,7 +5227,7 @@
       <x:c r="B16" t="str">
         <x:v>Pass. Patient.Blockchain_ID exists in schemas/dump and the migration maps seed patient IDs.</x:v>
       </x:c>
-      <x:c r="C16" s="48" t="str">
+      <x:c r="C16" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5125,7 +5238,7 @@
       <x:c r="B17" t="str">
         <x:v>Pass. node --check succeeded for backend/server.js and dental-backend/index.js; Vite frontend build passed with known warnings.</x:v>
       </x:c>
-      <x:c r="C17" s="48" t="str">
+      <x:c r="C17" s="56" t="str">
         <x:v>Pass (warnings)</x:v>
       </x:c>
     </x:row>
@@ -5136,7 +5249,7 @@
       <x:c r="B18" t="str">
         <x:v>Pass. /register now uses authorizeAdminRegistration and Signup.jsx sends jsonHeaders().</x:v>
       </x:c>
-      <x:c r="C18" s="48" t="str">
+      <x:c r="C18" s="56" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
@@ -5147,8 +5260,74 @@
       <x:c r="B19" t="str">
         <x:v>Pass. Deployment Migrations sheet tracks migration/env/smoke-test work for the existing AWS VM.</x:v>
       </x:c>
-      <x:c r="C19" s="48" t="str">
+      <x:c r="C19" s="56" t="str">
         <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>Phase 2 AWS Fabric deployment</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Pass. basic 1.0.1 sequence 3 committed with Org1MSP and Org2MSP approvals; PM2 Blockchain API restarted on role-bound identity selection.</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>Phase 2 live identity integration</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Pass. 9 direct gateway checks covered admin clinic scope, doctor actor scope, patient ownership, system logging, and violations.</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>Phase 2 chaincode unit tests</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Pass. 16 role, actor, clinic, system, missing MSP, and untrusted MSP tests completed on AWS temporary test workspace.</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Phase 2 gateway resolver tests</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Pass. 4 Node tests validated admin, doctor, patient, system, and missing-context wallet mappings.</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>AWS Phase 1 smoke tests 2026-07-11</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>Pass. Live AWS checks confirmed migration state, matching JWT secrets, restarted services, protected routes, admin access, doctor self-access, patient owner-only access, frontend availability, and protected registration.</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>AWS Phase 1 deployment gate</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Blocked on 2026-07-10. SSH reached edr.bizcenter.tech but the available local session has no accepted public key for ubuntu, so migration, env comparison, restart, and smoke tests were not executed.</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Blocked</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5164,7 +5343,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cdef8215d2f4a0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4044a855a294734"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5197,13 +5376,13 @@
       <x:c r="A3" s="16" t="s">
         <x:v>445</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>446</x:v>
+      <x:c r="B3" s="2" t="str">
+        <x:v>Phase 2 is deployed and verified on AWS. Remaining work is lifecycle automation for enrollment/revocation when clinics and users are added or removed.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="s">
-        <x:v>447</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
         <x:v>Mobile sign-in and request/consent calls now use JWT plus the login blockchainID; broader mobile screens still include static/placeholder workflows.</x:v>
@@ -5211,18 +5390,18 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="s">
         <x:v>448</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="s">
-        <x:v>449</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="s">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
         <x:v>450</x:v>
-      </x:c>
-      <x:c r="B6" s="2" t="s">
-        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5230,7 +5409,7 @@
         <x:v>Patient blockchain identity mapping</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Source-level mapping is implemented. AWS runtime databases must apply database/migrations/2026-07-10-add-patient-blockchain-id.sql before deploying the login query that selects Patient.Blockchain_ID.</x:v>
+        <x:v>Source-level mapping and AWS runtime verification passed 2026-07-11; Patient1-Patient3 mappings are present in the live database.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5238,7 +5417,7 @@
         <x:v>MSP/certificate token binding</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Phase 1 documents JWT as an API-session token signed with JWT_SECRET. User-specific MSP/certificate binding remains Phase 2 chaincode/gateway identity work.</x:v>
+        <x:v>Completed for current AWS identities on 2026-07-11. JWT claims select clinic/actor-bound X.509 wallet identities; ongoing enrollment/revocation automation remains a lifecycle item.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5249,10 +5428,18 @@
         <x:v>Source-level public registration is closed. AWS deployments must use an Admin/System JWT or set ADMIN_BOOTSTRAP_TOKEN temporarily for /register bootstrap.</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>AWS deployment access</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Phase 1 runtime gate is unverified. SSH to ubuntu@edr.bizcenter.tech currently fails with publickey authentication; obtain the deployment key or an authorized session before applying the migration or starting Phase 2.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069952b708e242e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d5cebf3e10f405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5270,22 +5457,22 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="46" t="str">
+      <x:c r="A1" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="46" t="str">
+      <x:c r="B1" s="53" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="C1" s="46" t="str">
+      <x:c r="C1" s="53" t="str">
         <x:v>Required On AWS VM</x:v>
       </x:c>
-      <x:c r="D1" s="46" t="str">
+      <x:c r="D1" s="53" t="str">
         <x:v>Source / Path</x:v>
       </x:c>
-      <x:c r="E1" s="46" t="str">
+      <x:c r="E1" s="53" t="str">
         <x:v>Action / Command</x:v>
       </x:c>
-      <x:c r="F1" s="46" t="str">
+      <x:c r="F1" s="53" t="str">
         <x:v>Status / Notes</x:v>
       </x:c>
     </x:row>
@@ -5306,7 +5493,7 @@
         <x:v>Run through MySQL client, then verify DESCRIBE Patient and Blockchain_ID backfill.</x:v>
       </x:c>
       <x:c r="F2" s="47" t="str">
-        <x:v>Pending remote execution; source migration file exists.</x:v>
+        <x:v>Passed 2026-07-11. Column and Patient1-Patient3 mappings already existed; rerun returned duplicate-column, so no destructive change was needed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5326,7 +5513,7 @@
         <x:v>Set the same strong JWT_SECRET in both APIs.</x:v>
       </x:c>
       <x:c r="F3" s="47" t="str">
-        <x:v>Pending remote confirmation.</x:v>
+        <x:v>Passed 2026-07-11. backend/.env and dental-backend/.env JWT_SECRET digests matched.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5346,7 +5533,7 @@
         <x:v>Set ADMIN_BOOTSTRAP_TOKEN, use it through x-bootstrap-token, then rotate/remove when no longer needed.</x:v>
       </x:c>
       <x:c r="F4" s="47" t="str">
-        <x:v>Pending remote decision.</x:v>
+        <x:v>Not enabled 2026-07-11. ADMIN_BOOTSTRAP_TOKEN is absent; bootstrap registration remains disabled.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -5366,7 +5553,232 @@
         <x:v>Execute checklist items 1-9 against the AWS VM.</x:v>
       </x:c>
       <x:c r="F5" s="47" t="str">
-        <x:v>Pending remote execution.</x:v>
+        <x:v>Passed 2026-07-11. Unauthenticated 401; admin 200; doctor cross-user 403; patient cross-user 403; frontend 200; anonymous registration 401.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="53" t="str">
+        <x:v>Change ID</x:v>
+      </x:c>
+      <x:c r="B1" s="53" t="str">
+        <x:v>Change / Control</x:v>
+      </x:c>
+      <x:c r="C1" s="53" t="str">
+        <x:v>Why This Change Was Required</x:v>
+      </x:c>
+      <x:c r="D1" s="53" t="str">
+        <x:v>SRS Gap Before Change</x:v>
+      </x:c>
+      <x:c r="E1" s="53" t="str">
+        <x:v>SRS Requirement(s) Addressed</x:v>
+      </x:c>
+      <x:c r="F1" s="53" t="str">
+        <x:v>Evidence / Result</x:v>
+      </x:c>
+      <x:c r="G1" s="53" t="str">
+        <x:v>Remaining SRS Limitation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="78" customHeight="1">
+      <x:c r="A2" s="55" t="str">
+        <x:v>P2-01</x:v>
+      </x:c>
+      <x:c r="B2" s="47" t="str">
+        <x:v>Chaincode MSP and RBAC enforcement</x:v>
+      </x:c>
+      <x:c r="C2" s="47" t="str">
+        <x:v>API JWT checks alone could be bypassed by invoking chaincode directly or through another gateway. Fabric therefore needed to enforce authorization at the ledger execution boundary.</x:v>
+      </x:c>
+      <x:c r="D2" s="47" t="str">
+        <x:v>Chaincode functions trusted the REST layer and did not consistently verify the invoking MSP, role, actor, clinic, ownership, assignment, or consent context.</x:v>
+      </x:c>
+      <x:c r="E2" s="47" t="str">
+        <x:v>SEC-02; SEC-06; FR-03; FR-13; FR-24; FR-25; FR-27</x:v>
+      </x:c>
+      <x:c r="F2" s="47" t="str">
+        <x:v>Implemented and deployed. Trusted Org1MSP/Org2MSP plus role, actorID, and clinicID attributes are validated by chaincode.</x:v>
+      </x:c>
+      <x:c r="G2" s="47" t="str">
+        <x:v>Automate enrollment/revocation as users and clinics are added or removed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="78" customHeight="1">
+      <x:c r="A3" s="55" t="str">
+        <x:v>P2-02</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="str">
+        <x:v>JWT-to-Fabric wallet identity binding</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>Transactions submitted as one shared appUser certificate could not prove which authenticated admin, doctor, patient, or system actor initiated the Fabric operation.</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>The Blockchain API used a shared Fabric identity, leaving an impersonation and non-repudiation gap even though API routes validated JWTs.</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>SEC-06; SEC-08; FR-24; FR-26</x:v>
+      </x:c>
+      <x:c r="F3" s="47" t="str">
+        <x:v>Implemented. JWT organization/blockchain claims select admin-, doctor-, patient-, or system-specific wallet identities; missing identities are rejected before gateway connection.</x:v>
+      </x:c>
+      <x:c r="G3" s="47" t="str">
+        <x:v>FR-02 remains a documented deviation: the API JWT itself is still signed with JWT_SECRET rather than an MSP certificate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="78" customHeight="1">
+      <x:c r="A4" s="55" t="str">
+        <x:v>P2-03</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="str">
+        <x:v>Role/actor-bound Fabric CA enrollment</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>Chaincode cannot make cryptographically grounded role and ownership decisions unless certificate attributes are issued and embedded by the Fabric CA.</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>The wallet contained only admin and shared appUser identities without the role, actorID, and admin clinicID attributes required by Phase 2 checks.</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>SEC-02; SEC-06; FR-03</x:v>
+      </x:c>
+      <x:c r="F4" s="47" t="str">
+        <x:v>Implemented on AWS. Clinic-bound admin, actor-bound doctor/patient, and system certificates were enrolled after backing up the wallet.</x:v>
+      </x:c>
+      <x:c r="G4" s="47" t="str">
+        <x:v>Identity issuance is currently an operational script, not yet integrated into database user lifecycle workflows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="78" customHeight="1">
+      <x:c r="A5" s="55" t="str">
+        <x:v>P2-04</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>Admin clinic-bound authorization</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>An Admin role by itself must not authorize an administrator from one clinic to manage or approve requests for another clinic.</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>Chaincode admin operations checked role but did not cryptographically bind the administrator to the target clinic.</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>FR-05 to FR-14; FR-22; FR-28; SEC-08</x:v>
+      </x:c>
+      <x:c r="F5" s="47" t="str">
+        <x:v>Implemented. Relevant patient/doctor management and request operations compare the transaction certificate clinicID with the requested clinic.</x:v>
+      </x:c>
+      <x:c r="G5" s="47" t="str">
+        <x:v>Full patient/doctor CRUD and notification workflow coverage remains in later phases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="78" customHeight="1">
+      <x:c r="A6" s="55" t="str">
+        <x:v>P2-05</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="str">
+        <x:v>Doctor actor, assignment, and consent checks</x:v>
+      </x:c>
+      <x:c r="C6" s="47" t="str">
+        <x:v>A doctor certificate must not impersonate another doctor or write/read clinical data for an unrelated patient.</x:v>
+      </x:c>
+      <x:c r="D6" s="47" t="str">
+        <x:v>Doctor-only role checks did not consistently enforce actorID, assigned-patient relationships, or granted sharing consent inside chaincode.</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>FR-13; FR-15; FR-16; FR-17; FR-21; FR-25; SEC-08</x:v>
+      </x:c>
+      <x:c r="F6" s="47" t="str">
+        <x:v>Implemented. Doctor identity, assignment, and consent are enforced for assigned-patient queries, requests, clinical records, dental data, and files.</x:v>
+      </x:c>
+      <x:c r="G6" s="47" t="str">
+        <x:v>Complete clinical REST/UI workflows and automatic access logging are still scheduled for later phases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="78" customHeight="1">
+      <x:c r="A7" s="55" t="str">
+        <x:v>P2-06</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="str">
+        <x:v>Patient owner-only chaincode paths</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>API owner checks were insufficient if a patient could call Fabric through another client or alter a transaction argument.</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
+        <x:v>Patient request, consent, and record transactions needed certificate actorID-to-patientID enforcement at chaincode level.</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
+        <x:v>FR-24; FR-27; SEC-02; SEC-06; SEC-08</x:v>
+      </x:c>
+      <x:c r="F7" s="47" t="str">
+        <x:v>Implemented. Patient certificate actorID must match the requested patient for consent, queues, records, dental data, and files.</x:v>
+      </x:c>
+      <x:c r="G7" s="47" t="str">
+        <x:v>Consent revocation, notifications, and full mobile workflow remain later-phase items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="78" customHeight="1">
+      <x:c r="A8" s="55" t="str">
+        <x:v>P2-07</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="str">
+        <x:v>System-only initialization and access logging</x:v>
+      </x:c>
+      <x:c r="C8" s="47" t="str">
+        <x:v>Ledger initialization and immutable audit creation are privileged service operations and must not be callable by ordinary users.</x:v>
+      </x:c>
+      <x:c r="D8" s="47" t="str">
+        <x:v>Initialization/helper functions were publicly invokable and LogAccess needed a dedicated service identity boundary.</x:v>
+      </x:c>
+      <x:c r="E8" s="47" t="str">
+        <x:v>FR-26; SEC-02; GDPR audit requirement</x:v>
+      </x:c>
+      <x:c r="F8" s="47" t="str">
+        <x:v>Implemented. System certificate is required for initialization and LogAccess; public actorExists is restricted to Admin/System.</x:v>
+      </x:c>
+      <x:c r="G8" s="47" t="str">
+        <x:v>Automatic LogAccess invocation on every approved data read remains Phase 8 work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="78" customHeight="1">
+      <x:c r="A9" s="55" t="str">
+        <x:v>P2-08</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="str">
+        <x:v>Role/MSP violation and live deployment evidence</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>Security controls require negative tests and deployed evidence; source inspection alone cannot prove enforcement across Fabric identities.</x:v>
+      </x:c>
+      <x:c r="D9" s="47" t="str">
+        <x:v>The SRS testing section required pass/fail evidence for unauthorized admin, doctor, patient, system, and MSP paths.</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
+        <x:v>SRS Section 8; SEC-02; SEC-06</x:v>
+      </x:c>
+      <x:c r="F9" s="47" t="str">
+        <x:v>Passed: 16 chaincode unit tests, 4 gateway resolver tests, 9 live identity checks, and AWS API regression smoke tests. Chaincode basic 1.0.1 sequence 3 is committed by both MSPs.</x:v>
+      </x:c>
+      <x:c r="G9" s="47" t="str">
+        <x:v>Performance, full workflow, and remaining FR evidence continue in Phase 12.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add Phase 3 SRS API parity
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6a6cecd44f2c4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="Rd434e3b4453b4baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="Rd9dfc3edc49a4c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rff780bfacbd24074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R53f729e8ab194b91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="Rd9185245136849c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R6bf5b8ad980f43d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R624e76df6fa84ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R7e797a0a71924a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="Rae6f27990a67483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="R0b40a4622ac64aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R3f9b5c634b304124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R0c16caa8558b47c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R2f1d101a53e2412a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1373,6 +1373,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="m/d/yy"/>
+  </x:numFmts>
   <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
@@ -1601,7 +1604,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1713,6 +1716,37 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2404,7 +2438,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R88eeefad4fa7410e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf9bbee3f7c2d4806"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2430,22 +2464,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RuntimeTable" displayName="RuntimeTable" ref="A1:E9" totalsRowShown="0" dataDxfId="14">
-  <x:autoFilter ref="A1:E9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RuntimeTable" displayName="RuntimeTable" ref="A1:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="14">
+  <x:autoFilter ref="A1:E10"/>
   <x:tableColumns count="5">
-    <x:tableColumn id="1" name="ID" dataDxfId="13"/>
-    <x:tableColumn id="2" name="Path" dataDxfId="18"/>
-    <x:tableColumn id="3" name="Type" dataDxfId="17"/>
-    <x:tableColumn id="4" name="What Changed" dataDxfId="16"/>
-    <x:tableColumn id="5" name="Purpose / Note" dataDxfId="15"/>
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Path"/>
+    <x:tableColumn id="3" name="Type"/>
+    <x:tableColumn id="4" name="What Changed"/>
+    <x:tableColumn id="5" name="Purpose / Note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VerificationTable" displayName="VerificationTable" ref="A1:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="9">
-  <x:autoFilter ref="A1:C25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VerificationTable" displayName="VerificationTable" ref="A1:C26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="9">
+  <x:autoFilter ref="A1:C26"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Verification Item"/>
     <x:tableColumn id="2" name="Result"/>
@@ -2456,8 +2490,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="KnownItemsTable" displayName="KnownItemsTable" ref="A1:B10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="1">
-  <x:autoFilter ref="A1:B10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="KnownItemsTable" displayName="KnownItemsTable" ref="A1:B11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0" dataDxfId="1">
+  <x:autoFilter ref="A1:B11"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Status / Note"/>
@@ -2703,8 +2737,8 @@
       <x:c r="A5" s="21" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B5" s="20" t="n">
-        <x:v>46213</x:v>
+      <x:c r="B5" s="57" t="n">
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2745,7 +2779,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="27" t="n">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2761,7 +2795,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="27" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2769,7 +2803,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="27" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2777,7 +2811,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="37" t="n">
-        <x:v>82</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2795,7 +2829,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B19" s="27" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2803,7 +2837,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B20" s="27" t="n">
-        <x:v>18</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2811,7 +2845,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B21" s="34" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2821,7 +2855,7 @@
     <x:mergeCell ref="A8:H8"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cc5b93e43b14815"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc990739613d47bf"/>
 </x:worksheet>
 </file>
 
@@ -4836,6 +4870,98 @@
       </x:c>
       <x:c r="G87" t="str">
         <x:v>Starts Phase 2 SEC-02 MSP enforcement after the AWS Phase 1 deployment gate passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>C-45</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>dental-backend/index.js</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Phase 3 route handlers</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>SRS Section 5 names were missing or mapped only to legacy routes; patient/doctor CRUD and role-specific rejection routes were not exposed.</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>Added all six SRS canonical routes, patient update/delete, doctor read/update/delete, separate admin/patient rejection, compatible alias metadata, and normalized canonical response envelopes.</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>Provides REST gateway parity while preserving existing clients and Phase 2 JWT-to-wallet identity binding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>C-46</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>Fabric / Chaincode</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>fabric-samples/dental-record-sharing/chaincode-javascript/lib/dentalRecordSharing.js</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>DeleteDoctor; DeletePatient</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>Delete transactions required Admin role but did not bind the admin certificate to the stored actor clinic.</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Delete transactions now load the stored doctor/patient and enforce _requireAdminClinic against its clinicID before deletion.</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>Preserves Phase 2 clinic/MSP isolation for the newly exposed delete APIs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>C-47</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>backend/server.js; dental-backend/index.js</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>JWT/role errors and canonical handlers</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>Authentication, authorization, validation, and Fabric errors used inconsistent flat error strings.</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>JWT/role failures now use a structured error object; canonical Blockchain API routes use success/data and success/error envelopes.</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>Makes errors predictable across Database and Blockchain APIs without changing legacy success payloads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>DOC-11</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>README.md; Outputs/SRS_Compliance_Base/*.md; Outputs/EDR_Remediation_Change_Log.md</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Phase 3 status and endpoint map</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>Phase 3 routes, aliases, roles, deployment requirements, and verification state were not documented.</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Documented exact canonical/legacy route mapping, roles, identity enforcement, source checks, no-DB-migration decision, and pending AWS rollout.</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Keeps roadmap, traceability, acceptance, startup context, and setup documentation synchronized.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4861,7 +4987,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac9f42c19ee8484a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3d3e2a978454db5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4876,163 +5002,180 @@
     <x:col min="4" max="5" width="61" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27.950000762939453" customHeight="1">
-      <x:c r="A1" s="13" t="s">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="58" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="s">
+      <x:c r="B1" s="58" t="s">
         <x:v>376</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="s">
+      <x:c r="C1" s="58" t="s">
         <x:v>377</x:v>
       </x:c>
-      <x:c r="D1" s="13" t="s">
+      <x:c r="D1" s="58" t="s">
         <x:v>378</x:v>
       </x:c>
-      <x:c r="E1" s="13" t="s">
+      <x:c r="E1" s="58" t="s">
         <x:v>379</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="3" t="s">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="59" t="s">
         <x:v>380</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="s">
+      <x:c r="B2" s="60" t="s">
         <x:v>381</x:v>
       </x:c>
-      <x:c r="C2" s="2" t="s">
+      <x:c r="C2" s="60" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="s">
+      <x:c r="D2" s="60" t="s">
         <x:v>383</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="s">
+      <x:c r="E2" s="60" t="s">
         <x:v>384</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="3" t="s">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="59" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="B3" s="60" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="s">
+      <x:c r="C3" s="60" t="s">
         <x:v>387</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
+      <x:c r="D3" s="60" t="s">
         <x:v>388</x:v>
       </x:c>
-      <x:c r="E3" s="2" t="s">
+      <x:c r="E3" s="60" t="s">
         <x:v>389</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="27">
-      <x:c r="A4" s="3" t="s">
+    <x:row r="4" ht="24" hidden="0" customHeight="1">
+      <x:c r="A4" s="59" t="s">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
+      <x:c r="B4" s="60" t="s">
         <x:v>391</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="C4" s="60" t="s">
         <x:v>392</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="D4" s="60" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="E4" s="60" t="s">
         <x:v>394</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="27">
-      <x:c r="A5" s="3" t="s">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="59" t="s">
         <x:v>395</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="s">
+      <x:c r="B5" s="60" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="C5" s="2" t="s">
+      <x:c r="C5" s="60" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="D5" s="2" t="s">
+      <x:c r="D5" s="60" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="E5" s="2" t="s">
+      <x:c r="E5" s="60" t="s">
         <x:v>399</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="3" t="s">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="59" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="s">
+      <x:c r="B6" s="60" t="s">
         <x:v>401</x:v>
       </x:c>
-      <x:c r="C6" s="2" t="s">
+      <x:c r="C6" s="60" t="s">
         <x:v>402</x:v>
       </x:c>
-      <x:c r="D6" s="2" t="s">
+      <x:c r="D6" s="60" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="E6" s="2" t="s">
+      <x:c r="E6" s="60" t="s">
         <x:v>404</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="27">
-      <x:c r="A7" s="3" t="s">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
+      <x:c r="A7" s="59" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="s">
+      <x:c r="B7" s="60" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="C7" s="2" t="s">
+      <x:c r="C7" s="60" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="D7" s="2" t="s">
+      <x:c r="D7" s="60" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="E7" s="2" t="s">
+      <x:c r="E7" s="60" t="s">
         <x:v>409</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="3" t="s">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="59" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="s">
+      <x:c r="B8" s="60" t="s">
         <x:v>411</x:v>
       </x:c>
-      <x:c r="C8" s="2" t="s">
+      <x:c r="C8" s="60" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="D8" s="2" t="s">
+      <x:c r="D8" s="60" t="s">
         <x:v>413</x:v>
       </x:c>
-      <x:c r="E8" s="2" t="s">
+      <x:c r="E8" s="60" t="s">
         <x:v>414</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="3" t="s">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="59" t="s">
         <x:v>415</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="s">
+      <x:c r="B9" s="60" t="s">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="C9" s="2" t="s">
+      <x:c r="C9" s="60" t="s">
         <x:v>417</x:v>
       </x:c>
-      <x:c r="D9" s="2" t="s">
+      <x:c r="D9" s="60" t="s">
         <x:v>418</x:v>
       </x:c>
-      <x:c r="E9" s="2" t="s">
+      <x:c r="E9" s="60" t="s">
         <x:v>419</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="61" t="str">
+        <x:v>R-09</x:v>
+      </x:c>
+      <x:c r="B10" s="61" t="str">
+        <x:v>/home/ubuntu/deployment-backups/20260711-094718</x:v>
+      </x:c>
+      <x:c r="C10" s="61" t="str">
+        <x:v>AWS deployment backup</x:v>
+      </x:c>
+      <x:c r="D10" s="61" t="str">
+        <x:v>Captured the pre-sync tracked diff, environment files, Compose override, Fabric connection profile, and wallet before resetting the VM checkout to commit 4892875.</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>Provides rollback evidence and preserves runtime identities/configuration for the Git-synchronized Phase 1 and Phase 2 deployment.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5debd18d7094971"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d65baa210294410"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5046,288 +5189,321 @@
     <x:col min="3" max="3" width="24.7109375" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27.950000762939453" customHeight="1">
-      <x:c r="A1" s="1" t="s">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="62" t="s">
         <x:v>420</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="s">
+      <x:c r="B1" s="62" t="s">
         <x:v>421</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="s">
+      <x:c r="C1" s="62" t="s">
         <x:v>422</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="2" t="s">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="60" t="s">
         <x:v>423</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="s">
+      <x:c r="B2" s="60" t="s">
         <x:v>424</x:v>
       </x:c>
-      <x:c r="C2" s="14" t="str">
+      <x:c r="C2" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B2)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="2" t="s">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="60" t="s">
         <x:v>425</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="B3" s="60" t="s">
         <x:v>426</x:v>
       </x:c>
-      <x:c r="C3" s="14" t="str">
+      <x:c r="C3" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B3)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="2" t="s">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="60" t="s">
         <x:v>427</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
+      <x:c r="B4" s="60" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="C4" s="14" t="str">
+      <x:c r="C4" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B4)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="2" t="s">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="60" t="s">
         <x:v>429</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="s">
+      <x:c r="B5" s="60" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="C5" s="14" t="str">
+      <x:c r="C5" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B5)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="2" t="s">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="60" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="s">
+      <x:c r="B6" s="60" t="s">
         <x:v>432</x:v>
       </x:c>
-      <x:c r="C6" s="14" t="str">
+      <x:c r="C6" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B6)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="2" t="s">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="60" t="s">
         <x:v>433</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="s">
+      <x:c r="B7" s="60" t="s">
         <x:v>434</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
+      <x:c r="C7" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B7)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="2" t="s">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="60" t="s">
         <x:v>435</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="s">
+      <x:c r="B8" s="60" t="s">
         <x:v>436</x:v>
       </x:c>
-      <x:c r="C8" s="14" t="str">
+      <x:c r="C8" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B8)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="27">
-      <x:c r="A9" s="2" t="s">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="60" t="s">
         <x:v>437</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="s">
+      <x:c r="B9" s="60" t="s">
         <x:v>438</x:v>
       </x:c>
-      <x:c r="C9" s="14" t="str">
+      <x:c r="C9" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B9)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="2" t="s">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="60" t="s">
         <x:v>439</x:v>
       </x:c>
-      <x:c r="B10" s="2" t="s">
+      <x:c r="B10" s="60" t="s">
         <x:v>440</x:v>
       </x:c>
-      <x:c r="C10" s="14" t="str">
+      <x:c r="C10" s="63" t="str">
         <x:f>IF(ISNUMBER(SEARCH("warning",B10)),"Pass (warnings)","Pass")</x:f>
         <x:v>Pass (warnings)</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="61" t="str">
         <x:v>Phase 1 server syntax checks</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B11" s="61" t="str">
         <x:v>Pass. node --check succeeded for backend/server.js and dental-backend/index.js.</x:v>
       </x:c>
-      <x:c r="C11" s="56" t="str">
+      <x:c r="C11" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="61" t="str">
         <x:v>Blockchain API package metadata</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B12" s="61" t="str">
         <x:v>Pass. package.json and package-lock.json parse after adding jsonwebtoken.</x:v>
       </x:c>
-      <x:c r="C12" s="56" t="str">
+      <x:c r="C12" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="61" t="str">
         <x:v>Mobile hard-coded protected request scan</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="61" t="str">
         <x:v>Pass. No active Patient1/API_BASE_URL protected request calls found.</x:v>
       </x:c>
-      <x:c r="C13" s="56" t="str">
+      <x:c r="C13" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="61" t="str">
         <x:v>Patient identity syntax checks</x:v>
       </x:c>
-      <x:c r="B14" t="str">
+      <x:c r="B14" s="61" t="str">
         <x:v>Pass. node --check succeeded for backend/server.js, dental-backend/index.js, and BC-Dentistry-Mobile-App/utils/api.js.</x:v>
       </x:c>
-      <x:c r="C14" s="56" t="str">
+      <x:c r="C14" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="61" t="str">
         <x:v>Patient owner-route scan</x:v>
       </x:c>
-      <x:c r="B15" t="str">
+      <x:c r="B15" s="61" t="str">
         <x:v>Pass. requirePatientSelfParam/body middleware is applied to patient request and consent routes.</x:v>
       </x:c>
-      <x:c r="C15" s="56" t="str">
+      <x:c r="C15" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="61" t="str">
         <x:v>Patient mapping schema scan</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="B16" s="61" t="str">
         <x:v>Pass. Patient.Blockchain_ID exists in schemas/dump and the migration maps seed patient IDs.</x:v>
       </x:c>
-      <x:c r="C16" s="56" t="str">
+      <x:c r="C16" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="61" t="str">
         <x:v>Phase 1 bootstrap syntax/build checks</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B17" s="61" t="str">
         <x:v>Pass. node --check succeeded for backend/server.js and dental-backend/index.js; Vite frontend build passed with known warnings.</x:v>
       </x:c>
-      <x:c r="C17" s="56" t="str">
+      <x:c r="C17" s="64" t="str">
         <x:v>Pass (warnings)</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="61" t="str">
         <x:v>Protected registration scan</x:v>
       </x:c>
-      <x:c r="B18" t="str">
+      <x:c r="B18" s="61" t="str">
         <x:v>Pass. /register now uses authorizeAdminRegistration and Signup.jsx sends jsonHeaders().</x:v>
       </x:c>
-      <x:c r="C18" s="56" t="str">
+      <x:c r="C18" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="61" t="str">
         <x:v>AWS migration tracker</x:v>
       </x:c>
-      <x:c r="B19" t="str">
+      <x:c r="B19" s="61" t="str">
         <x:v>Pass. Deployment Migrations sheet tracks migration/env/smoke-test work for the existing AWS VM.</x:v>
       </x:c>
-      <x:c r="C19" s="56" t="str">
+      <x:c r="C19" s="64" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="61" t="str">
         <x:v>Phase 2 AWS Fabric deployment</x:v>
       </x:c>
-      <x:c r="B20" t="str">
+      <x:c r="B20" s="61" t="str">
         <x:v>Pass. basic 1.0.1 sequence 3 committed with Org1MSP and Org2MSP approvals; PM2 Blockchain API restarted on role-bound identity selection.</x:v>
       </x:c>
-      <x:c r="C20" t="str">
+      <x:c r="C20" s="61" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="str">
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="61" t="str">
         <x:v>Phase 2 live identity integration</x:v>
       </x:c>
-      <x:c r="B21" t="str">
+      <x:c r="B21" s="61" t="str">
         <x:v>Pass. 9 direct gateway checks covered admin clinic scope, doctor actor scope, patient ownership, system logging, and violations.</x:v>
       </x:c>
-      <x:c r="C21" t="str">
+      <x:c r="C21" s="61" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="61" t="str">
         <x:v>Phase 2 chaincode unit tests</x:v>
       </x:c>
-      <x:c r="B22" t="str">
+      <x:c r="B22" s="61" t="str">
         <x:v>Pass. 16 role, actor, clinic, system, missing MSP, and untrusted MSP tests completed on AWS temporary test workspace.</x:v>
       </x:c>
-      <x:c r="C22" t="str">
+      <x:c r="C22" s="61" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="str">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="61" t="str">
         <x:v>Phase 2 gateway resolver tests</x:v>
       </x:c>
-      <x:c r="B23" t="str">
+      <x:c r="B23" s="61" t="str">
         <x:v>Pass. 4 Node tests validated admin, doctor, patient, system, and missing-context wallet mappings.</x:v>
       </x:c>
-      <x:c r="C23" t="str">
+      <x:c r="C23" s="61" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="str">
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A24" s="61" t="str">
         <x:v>AWS Phase 1 smoke tests 2026-07-11</x:v>
       </x:c>
-      <x:c r="B24" t="str">
+      <x:c r="B24" s="61" t="str">
         <x:v>Pass. Live AWS checks confirmed migration state, matching JWT secrets, restarted services, protected routes, admin access, doctor self-access, patient owner-only access, frontend availability, and protected registration.</x:v>
       </x:c>
-      <x:c r="C24" t="str">
+      <x:c r="C24" s="61" t="str">
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" t="str">
-        <x:v>AWS Phase 1 deployment gate</x:v>
-      </x:c>
-      <x:c r="B25" t="str">
-        <x:v>Blocked on 2026-07-10. SSH reached edr.bizcenter.tech but the available local session has no accepted public key for ubuntu, so migration, env comparison, restart, and smoke tests were not executed.</x:v>
-      </x:c>
-      <x:c r="C25" t="str">
-        <x:v>Blocked</x:v>
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="61" t="str">
+        <x:v>AWS Git-synchronized Phase 1/2 redeployment 2026-07-11</x:v>
+      </x:c>
+      <x:c r="B25" s="61" t="str">
+        <x:v>Pass. VM checkout aligned to commit 4892875; Database API rebuilt, Blockchain API restarted, frontend rebuilt/copied to Nginx, JWT secrets matched, bootstrap token remained absent, patient mappings were verified, and public smoke tests passed.</x:v>
+      </x:c>
+      <x:c r="C25" s="61" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A26" s="61" t="str">
+        <x:v>Chaincode test execution after Git sync</x:v>
+      </x:c>
+      <x:c r="B26" s="61" t="str">
+        <x:v>Pass with known tooling issue. All 16 Mocha chaincode checks passed when invoked directly. The npm test pre-hook still fails because the inherited ESLint parser configuration does not parse object spread syntax used by the Node 18+ source.</x:v>
+      </x:c>
+      <x:c r="C26" s="61" t="str">
+        <x:v>Pass (warnings)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>Phase 3 API syntax and route/RBAC suite</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Pass. Database and Blockchain API syntax checks passed; 7 identity resolver and Phase 3 route/JWT/role/envelope tests passed.</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>Phase 3 AWS deployment and smoke test</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Pending. SSH endpoint was reachable on 2026-07-11, but the available session credentials were rejected. Do not mark deployed until Blockchain API, chaincode, canonical routes, and aliases pass live smoke tests.</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Pending</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5343,7 +5519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4044a855a294734"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcc704ecd7ee4c71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5356,90 +5532,106 @@
     <x:col min="2" max="2" width="118.140625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="27.950000762939453" customHeight="1">
-      <x:c r="A1" s="15" t="s">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="65" t="s">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="B1" s="15" t="s">
+      <x:c r="B1" s="65" t="s">
         <x:v>442</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="16" t="s">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="66" t="s">
         <x:v>443</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="s">
+      <x:c r="B2" s="60" t="s">
         <x:v>444</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="16" t="s">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="66" t="s">
         <x:v>445</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="str">
+      <x:c r="B3" s="60" t="str">
         <x:v>Phase 2 is deployed and verified on AWS. Remaining work is lifecycle automation for enrollment/revocation when clinics and users are added or removed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="16" t="s">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="66" t="s">
         <x:v>446</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="str">
+      <x:c r="B4" s="60" t="str">
         <x:v>Mobile sign-in and request/consent calls now use JWT plus the login blockchainID; broader mobile screens still include static/placeholder workflows.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="16" t="s">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="66" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="s">
+      <x:c r="B5" s="60" t="s">
         <x:v>448</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="16" t="s">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="66" t="s">
         <x:v>449</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="s">
+      <x:c r="B6" s="60" t="s">
         <x:v>450</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="61" t="str">
         <x:v>Patient blockchain identity mapping</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c r="B7" s="61" t="str">
         <x:v>Source-level mapping and AWS runtime verification passed 2026-07-11; Patient1-Patient3 mappings are present in the live database.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="61" t="str">
         <x:v>MSP/certificate token binding</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c r="B8" s="61" t="str">
         <x:v>Completed for current AWS identities on 2026-07-11. JWT claims select clinic/actor-bound X.509 wallet identities; ongoing enrollment/revocation automation remains a lifecycle item.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="61" t="str">
         <x:v>Bootstrap admin registration</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B9" s="61" t="str">
         <x:v>Source-level public registration is closed. AWS deployments must use an Admin/System JWT or set ADMIN_BOOTSTRAP_TOKEN temporarily for /register bootstrap.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>AWS deployment access</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Phase 1 runtime gate is unverified. SSH to ubuntu@edr.bizcenter.tech currently fails with publickey authentication; obtain the deployment key or an authorized session before applying the migration or starting Phase 2.</x:v>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="61" t="str">
+        <x:v>Chaincode lint pre-hook</x:v>
+      </x:c>
+      <x:c r="B10" s="61" t="str">
+        <x:v>The deployed chaincode and all 16 direct Mocha tests pass, but npm test stops in the inherited ESLint pre-hook at object spread syntax. Update the ESLint parser/ecmaVersion configuration so the standard npm test command can run end to end.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="61" t="str">
+        <x:v>Dependency audit findings</x:v>
+      </x:c>
+      <x:c r="B11" s="61" t="str">
+        <x:v>Clean AWS installs reported existing npm audit findings: dental-backend 28 vulnerabilities (3 critical), frontend 33 (1 critical), and chaincode 19 (1 critical). Review and remediate with compatibility testing; do not apply npm audit fix --force directly to production.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Phase 3 AWS rollout pending</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>No DB migration is required. Deploy/restart dental-backend; package, approve, and commit the clinic-scoped delete chaincode update; then run JWT/role/identity smoke tests for every canonical endpoint and legacy alias.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d5cebf3e10f405e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b55f38fa3f842e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5456,27 +5648,27 @@
     <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="53" t="str">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="46" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="53" t="str">
+      <x:c r="B1" s="46" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="C1" s="53" t="str">
+      <x:c r="C1" s="46" t="str">
         <x:v>Required On AWS VM</x:v>
       </x:c>
-      <x:c r="D1" s="53" t="str">
+      <x:c r="D1" s="46" t="str">
         <x:v>Source / Path</x:v>
       </x:c>
-      <x:c r="E1" s="53" t="str">
+      <x:c r="E1" s="46" t="str">
         <x:v>Action / Command</x:v>
       </x:c>
-      <x:c r="F1" s="53" t="str">
+      <x:c r="F1" s="46" t="str">
         <x:v>Status / Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A2" s="47" t="str">
         <x:v>MIG-01</x:v>
       </x:c>
@@ -5496,7 +5688,7 @@
         <x:v>Passed 2026-07-11. Column and Patient1-Patient3 mappings already existed; rerun returned duplicate-column, so no destructive change was needed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A3" s="47" t="str">
         <x:v>ENV-01</x:v>
       </x:c>
@@ -5516,7 +5708,7 @@
         <x:v>Passed 2026-07-11. backend/.env and dental-backend/.env JWT_SECRET digests matched.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="47" t="str">
         <x:v>ENV-02</x:v>
       </x:c>
@@ -5536,7 +5728,7 @@
         <x:v>Not enabled 2026-07-11. ADMIN_BOOTSTRAP_TOKEN is absent; bootstrap registration remains disabled.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A5" s="47" t="str">
         <x:v>TEST-01</x:v>
       </x:c>
@@ -5553,7 +5745,27 @@
         <x:v>Execute checklist items 1-9 against the AWS VM.</x:v>
       </x:c>
       <x:c r="F5" s="47" t="str">
-        <x:v>Passed 2026-07-11. Unauthenticated 401; admin 200; doctor cross-user 403; patient cross-user 403; frontend 200; anonymous registration 401.</x:v>
+        <x:v>Passed again after Git sync on 2026-07-11 at commit 4892875. Public checks: frontend 200; unauthenticated Database/Blockchain APIs 401; admin paths 200; doctor and patient cross-identity paths 403; anonymous registration 401; authorized invalid registration reached 400 validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="78" customHeight="1">
+      <x:c r="A6" s="61" t="str">
+        <x:v>P3-DEP-01</x:v>
+      </x:c>
+      <x:c r="B6" s="61" t="str">
+        <x:v>Phase 3 REST API and chaincode rollout</x:v>
+      </x:c>
+      <x:c r="C6" s="61" t="str">
+        <x:v>No database migration</x:v>
+      </x:c>
+      <x:c r="D6" s="61" t="str">
+        <x:v>Deploy dental-backend and commit updated basic chaincode sequence; restart PM2 service.</x:v>
+      </x:c>
+      <x:c r="E6" s="61" t="str">
+        <x:v>Smoke-test all canonical routes, legacy aliases, 401/403 role cases, doctor/patient actor mismatch, and admin clinic mismatch.</x:v>
+      </x:c>
+      <x:c r="F6" s="61" t="str">
+        <x:v>Pending - AWS SSH key not accepted in current session</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5574,31 +5786,31 @@
     <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="53" t="str">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="46" t="str">
         <x:v>Change ID</x:v>
       </x:c>
-      <x:c r="B1" s="53" t="str">
+      <x:c r="B1" s="46" t="str">
         <x:v>Change / Control</x:v>
       </x:c>
-      <x:c r="C1" s="53" t="str">
+      <x:c r="C1" s="46" t="str">
         <x:v>Why This Change Was Required</x:v>
       </x:c>
-      <x:c r="D1" s="53" t="str">
+      <x:c r="D1" s="46" t="str">
         <x:v>SRS Gap Before Change</x:v>
       </x:c>
-      <x:c r="E1" s="53" t="str">
+      <x:c r="E1" s="46" t="str">
         <x:v>SRS Requirement(s) Addressed</x:v>
       </x:c>
-      <x:c r="F1" s="53" t="str">
+      <x:c r="F1" s="46" t="str">
         <x:v>Evidence / Result</x:v>
       </x:c>
-      <x:c r="G1" s="53" t="str">
+      <x:c r="G1" s="46" t="str">
         <x:v>Remaining SRS Limitation</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="78" customHeight="1">
-      <x:c r="A2" s="55" t="str">
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A2" s="67" t="str">
         <x:v>P2-01</x:v>
       </x:c>
       <x:c r="B2" s="47" t="str">
@@ -5620,8 +5832,8 @@
         <x:v>Automate enrollment/revocation as users and clinics are added or removed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="78" customHeight="1">
-      <x:c r="A3" s="55" t="str">
+    <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A3" s="67" t="str">
         <x:v>P2-02</x:v>
       </x:c>
       <x:c r="B3" s="47" t="str">
@@ -5643,8 +5855,8 @@
         <x:v>FR-02 remains a documented deviation: the API JWT itself is still signed with JWT_SECRET rather than an MSP certificate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="78" customHeight="1">
-      <x:c r="A4" s="55" t="str">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A4" s="67" t="str">
         <x:v>P2-03</x:v>
       </x:c>
       <x:c r="B4" s="47" t="str">
@@ -5666,8 +5878,8 @@
         <x:v>Identity issuance is currently an operational script, not yet integrated into database user lifecycle workflows.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="78" customHeight="1">
-      <x:c r="A5" s="55" t="str">
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A5" s="67" t="str">
         <x:v>P2-04</x:v>
       </x:c>
       <x:c r="B5" s="47" t="str">
@@ -5689,8 +5901,8 @@
         <x:v>Full patient/doctor CRUD and notification workflow coverage remains in later phases.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="78" customHeight="1">
-      <x:c r="A6" s="55" t="str">
+    <x:row r="6" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A6" s="67" t="str">
         <x:v>P2-05</x:v>
       </x:c>
       <x:c r="B6" s="47" t="str">
@@ -5712,8 +5924,8 @@
         <x:v>Complete clinical REST/UI workflows and automatic access logging are still scheduled for later phases.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="78" customHeight="1">
-      <x:c r="A7" s="55" t="str">
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="67" t="str">
         <x:v>P2-06</x:v>
       </x:c>
       <x:c r="B7" s="47" t="str">
@@ -5735,8 +5947,8 @@
         <x:v>Consent revocation, notifications, and full mobile workflow remain later-phase items.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="78" customHeight="1">
-      <x:c r="A8" s="55" t="str">
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="67" t="str">
         <x:v>P2-07</x:v>
       </x:c>
       <x:c r="B8" s="47" t="str">
@@ -5758,8 +5970,8 @@
         <x:v>Automatic LogAccess invocation on every approved data read remains Phase 8 work.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="78" customHeight="1">
-      <x:c r="A9" s="55" t="str">
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
+      <x:c r="A9" s="67" t="str">
         <x:v>P2-08</x:v>
       </x:c>
       <x:c r="B9" s="47" t="str">
@@ -5775,10 +5987,33 @@
         <x:v>SRS Section 8; SEC-02; SEC-06</x:v>
       </x:c>
       <x:c r="F9" s="47" t="str">
-        <x:v>Passed: 16 chaincode unit tests, 4 gateway resolver tests, 9 live identity checks, and AWS API regression smoke tests. Chaincode basic 1.0.1 sequence 3 is committed by both MSPs.</x:v>
+        <x:v>Passed after Git-synchronized redeployment of commit 4892875: 16 direct chaincode tests, 4 gateway resolver tests, 9 live Fabric identity checks, and the full AWS API regression smoke suite. Chaincode basic 1.0.1 sequence 3 remains committed by Org1MSP and Org2MSP.</x:v>
       </x:c>
       <x:c r="G9" s="47" t="str">
         <x:v>Performance, full workflow, and remaining FR evidence continue in Phase 12.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>SRS Section 5 API gateway parity</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Phase 3</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Implemented at source</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>dental-backend/index.js; phase3RouteParity.test.js</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Six canonical routes, patient/doctor CRUD, separate reject routes, normalized envelopes</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>7/7 route/identity tests pass; syntax checks pass</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>AWS deployment pending</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Complete Phase 4 patient management
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc3bd67fe642b4080"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R5b314ad488274a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="Rbe43d9f90321443d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="R9dfa49224c8642dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="Ra7a03369eed24136"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R9df11f6551ad456a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R947a7657488c4413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re533bdf1e175412a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="Rf179ebb55fac4df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R3bfd9c82e04c47b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rf367a5505cee4d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R52b697199a814f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R0990df66580345fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R3ca4e1db49554cef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3385,7 +3385,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra607054e34d8465a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R032d6b3edf864804"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3685,7 +3685,7 @@
       <x:c r="B6" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C6" s="17">
+      <x:c r="C6" s="17" t="n">
         <x:v>46214</x:v>
       </x:c>
     </x:row>
@@ -3838,7 +3838,7 @@
     <x:mergeCell ref="B9:I9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R709adf9b63f144e8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d27d312e53f4bd1"/>
 </x:worksheet>
 </file>
 
@@ -5947,6 +5947,144 @@
       </x:c>
       <x:c r="G91" s="43" t="s">
         <x:v>511</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>C-91</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>backend/server.js</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Phase 4 patient management</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Patient data was primarily read from Fabric and CRUD was incomplete.</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Added JWT/admin/clinic-bound hybrid create, list, owner/admin read, update, assignment, and coordinated delete routes with validation, UUID IDs, transactions and SHA-256.</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>Completes FR-05 to FR-10 while keeping PII off-chain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>C-92</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>database/dump.sql; database/migrations/2026-07-11-phase4-patient-management.sql</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Patient table Phase 4 fields</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Patient table held DOB, gender, Emirates ID and blockchain mapping only.</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Added nationality, address, blood type, JSON medical history/allergies/medications/insurance/doctors, clinic, modified date, uniqueness and clinic index/FK.</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Makes MySQL authoritative for detailed patient PII and clinical/admin data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>C-93</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>Fabric / Chaincode</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>fabric-samples/dental-record-sharing/chaincode-javascript/lib/dentalRecordSharing.js</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>AddPatientMetadata; UpdatePatientMetadata</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Patient transactions stored names, Emirates ID, email, contact and address on-chain.</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Added metadata-only transactions storing IDs, clinic/doctors, opaque MySQL reference, SHA-256 hash, timestamps and storage policy.</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Aligns new patient writes with SEC-03; historical ledger PII cleanup remains a deployment gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>C-94</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>dental-backend/index.js</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>/patient-metadata routes</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>No metadata-only patient gateway routes existed.</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Added JWT admin-only, clinic-bound create/update/delete metadata routes mapped to Fabric identities.</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>Preserves Phase 1 JWT and Phase 2 MSP/RBAC binding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>C-95</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>bc-dentistry-frontend/src/assets/components/Patients; assets/Pages/Patients.jsx</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Phase 4 patient UI</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Add form omitted functioning medical/insurance fields and had no update/assign/delete workflow.</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Added complete SRS add form, MySQL list integration, update and assignment actions, and confirmed delete with surfaced errors.</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Completes admin patient-management workflow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>C-96</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Tests / Deployment</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>dental-backend/test/phase4PatientManagement.test.js</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>3 tests</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>No Phase 4 source assertions.</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Added route, hybrid-storage and authorization assertions; 10 total Phase 2-4 tests pass.</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Protects API coverage and SEC-03 design.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5987,7 +6125,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a7c32b0810e4259"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7041ad5563334f85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6177,7 +6315,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83a637c6425b46ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5db5c180376429a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6498,6 +6636,39 @@
       </x:c>
       <x:c r="C28" s="49" t="str">
         <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>V-28</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Phase 4 Node syntax</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Passed: backend, Blockchain API and chaincode parse with bundled Node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>V-29</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>Phase 2-4 route/identity tests</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Passed: 10/10 Node tests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>V-30</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Frontend production build</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Passed: Vite 5.3.3 production build completed (1,904 modules). Existing unresolved font and large-chunk warnings remain non-blocking.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6518,7 +6689,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R857961ab23204b6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bf2a89aaf62490c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6631,7 +6802,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ad1a57f3f6149b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44441e59a084a43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6767,6 +6938,66 @@
       </x:c>
       <x:c r="F6" s="45" t="str">
         <x:v>Passed 2026-07-11. AWS checkout b30cae6; PM2 Blockchain API online; basic 1.0.2 sequence 4 committed with Org1MSP/Org2MSP approvals; 13 authenticated smoke checks passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>P4-DB-01</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Database migration</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Yes, before Phase 4 Database API restart</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Source_Code_Remediation/database/migrations/2026-07-11-phase4-patient-management.sql</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Back up MySQL; apply migration; DESCRIBE Patient; verify unique Emirates_ID and clinic FK/index.</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Pending AWS deployment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>P4-FAB-01</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Fabric chaincode upgrade</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>dentalRecordSharing.js AddPatientMetadata/UpdatePatientMetadata</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Package/install/approve/commit next basic version and sequence; sanitize historical patient state containing PII.</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Pending AWS deployment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>P4-APP-01</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>API/frontend rollout</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Yes, after DB and Fabric</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>backend, dental-backend, bc-dentistry-frontend</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Restart both PM2 APIs; clean-install/build frontend; copy dist to /var/www/edr; run authenticated create/update/read/assign/delete and negative role/clinic/owner smoke tests.</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Pending AWS deployment.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7018,6 +7249,44 @@
         <x:v>Complete</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>P4-FR05-10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>FR-05 to FR-10</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Source complete</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Hybrid patient CRUD/assignment with all SRS fields, UUID and UI actions.</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>AWS deploy and smoke validation pending.</x:v>
+      </x:c>
+      <x:c r="F11" t="str"/>
+      <x:c r="G11" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>P4-SEC03</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>SEC-03</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Source complete for new patient writes</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>MySQL PII plus Fabric reference/SHA-256 metadata only.</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Historical patient ledger PII cleanup and Phase 5 doctor split pending.</x:v>
+      </x:c>
+      <x:c r="F12" t="str"/>
+      <x:c r="G12" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Classify remediation work against SRS gaps
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re533bdf1e175412a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="Rf179ebb55fac4df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R3bfd9c82e04c47b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rf367a5505cee4d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R52b697199a814f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R0990df66580345fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R3ca4e1db49554cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rae105639453d4165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R13a19759e0ca4016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="Rde9bfb0fd3294612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="R4be189abdf594137"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R4164590d035347b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R212cb54529034869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R0f311e4fed564dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="R57ec69ca88854dc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2225,10 +2226,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="m/d/yy"/>
+    <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -2357,8 +2359,20 @@
       <x:color rgb="FF215868"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2450,8 +2464,38 @@
         <x:fgColor rgb="FFDAEEF3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1F3A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1F3A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="15">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -2493,11 +2537,101 @@
         <x:color rgb="FFD9D9D9"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="108">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2627,6 +2761,108 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -3385,7 +3621,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R032d6b3edf864804"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ec74262157141e9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3838,7 +4074,7 @@
     <x:mergeCell ref="B9:I9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d27d312e53f4bd1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e99b74393c24f4c"/>
 </x:worksheet>
 </file>
 
@@ -3854,6 +4090,10 @@
     <x:col min="6" max="6" width="81.42578125" style="30" customWidth="1"/>
     <x:col min="7" max="7" width="99.7109375" style="30" customWidth="1"/>
     <x:col min="8" max="16384" width="9.140625" style="30" customWidth="0"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3878,6 +4118,18 @@
       <x:c r="G1" s="22" t="s">
         <x:v>28</x:v>
       </x:c>
+      <x:c r="H1" t="str">
+        <x:v>Work Type</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>Remediation Phase</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>SRS Requirement / Scope</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>Classification Basis</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="27">
       <x:c r="A2" s="31" t="s">
@@ -3901,6 +4153,18 @@
       <x:c r="G2" s="33" t="s">
         <x:v>34</x:v>
       </x:c>
+      <x:c r="H2" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I2" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J2" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K2" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="31" t="s">
@@ -3924,6 +4188,18 @@
       <x:c r="G3" s="33" t="s">
         <x:v>39</x:v>
       </x:c>
+      <x:c r="H3" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I3" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J3" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K3" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="27">
       <x:c r="A4" s="31" t="s">
@@ -3947,6 +4223,18 @@
       <x:c r="G4" s="33" t="s">
         <x:v>44</x:v>
       </x:c>
+      <x:c r="H4" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I4" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J4" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K4" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="40.5">
       <x:c r="A5" s="31" t="s">
@@ -3970,6 +4258,18 @@
       <x:c r="G5" s="33" t="s">
         <x:v>49</x:v>
       </x:c>
+      <x:c r="H5" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I5" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J5" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K5" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="40.5">
       <x:c r="A6" s="31" t="s">
@@ -3993,6 +4293,18 @@
       <x:c r="G6" s="33" t="s">
         <x:v>55</x:v>
       </x:c>
+      <x:c r="H6" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I6" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J6" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K6" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="31" t="s">
@@ -4016,6 +4328,18 @@
       <x:c r="G7" s="33" t="s">
         <x:v>60</x:v>
       </x:c>
+      <x:c r="H7" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I7" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J7" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K7" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="27">
       <x:c r="A8" s="31" t="s">
@@ -4039,6 +4363,18 @@
       <x:c r="G8" s="33" t="s">
         <x:v>65</x:v>
       </x:c>
+      <x:c r="H8" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I8" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J8" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K8" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="27">
       <x:c r="A9" s="31" t="s">
@@ -4062,6 +4398,18 @@
       <x:c r="G9" s="33" t="s">
         <x:v>70</x:v>
       </x:c>
+      <x:c r="H9" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I9" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J9" s="56" t="str">
+        <x:v>FR-05; FR-06</x:v>
+      </x:c>
+      <x:c r="K9" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="27">
       <x:c r="A10" s="31" t="s">
@@ -4085,6 +4433,18 @@
       <x:c r="G10" s="33" t="s">
         <x:v>75</x:v>
       </x:c>
+      <x:c r="H10" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I10" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J10" s="56" t="str">
+        <x:v>FR-11</x:v>
+      </x:c>
+      <x:c r="K10" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="31" t="s">
@@ -4108,6 +4468,18 @@
       <x:c r="G11" s="33" t="s">
         <x:v>80</x:v>
       </x:c>
+      <x:c r="H11" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I11" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J11" s="56" t="str">
+        <x:v>FR-09; FR-13</x:v>
+      </x:c>
+      <x:c r="K11" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="27">
       <x:c r="A12" s="31" t="s">
@@ -4131,6 +4503,18 @@
       <x:c r="G12" s="33" t="s">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="H12" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I12" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J12" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K12" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="27">
       <x:c r="A13" s="31" t="s">
@@ -4154,6 +4538,18 @@
       <x:c r="G13" s="33" t="s">
         <x:v>91</x:v>
       </x:c>
+      <x:c r="H13" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I13" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J13" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K13" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="27">
       <x:c r="A14" s="31" t="s">
@@ -4177,6 +4573,18 @@
       <x:c r="G14" s="33" t="s">
         <x:v>96</x:v>
       </x:c>
+      <x:c r="H14" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I14" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J14" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K14" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="27">
       <x:c r="A15" s="31" t="s">
@@ -4200,6 +4608,18 @@
       <x:c r="G15" s="33" t="s">
         <x:v>101</x:v>
       </x:c>
+      <x:c r="H15" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I15" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J15" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K15" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="27">
       <x:c r="A16" s="31" t="s">
@@ -4223,6 +4643,18 @@
       <x:c r="G16" s="33" t="s">
         <x:v>105</x:v>
       </x:c>
+      <x:c r="H16" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I16" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J16" s="56" t="str">
+        <x:v>FR-27</x:v>
+      </x:c>
+      <x:c r="K16" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="27">
       <x:c r="A17" s="31" t="s">
@@ -4246,6 +4678,18 @@
       <x:c r="G17" s="33" t="s">
         <x:v>110</x:v>
       </x:c>
+      <x:c r="H17" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I17" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J17" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K17" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="27">
       <x:c r="A18" s="31" t="s">
@@ -4269,6 +4713,18 @@
       <x:c r="G18" s="33" t="s">
         <x:v>115</x:v>
       </x:c>
+      <x:c r="H18" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I18" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J18" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K18" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="27">
       <x:c r="A19" s="31" t="s">
@@ -4292,6 +4748,18 @@
       <x:c r="G19" s="33" t="s">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="H19" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I19" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J19" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K19" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="s">
@@ -4315,6 +4783,18 @@
       <x:c r="G20" s="33" t="s">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="H20" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I20" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J20" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K20" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="27">
       <x:c r="A21" s="31" t="s">
@@ -4338,6 +4818,18 @@
       <x:c r="G21" s="33" t="s">
         <x:v>130</x:v>
       </x:c>
+      <x:c r="H21" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I21" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J21" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K21" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="27">
       <x:c r="A22" s="31" t="s">
@@ -4361,6 +4853,18 @@
       <x:c r="G22" s="33" t="s">
         <x:v>136</x:v>
       </x:c>
+      <x:c r="H22" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I22" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J22" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K22" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="27">
       <x:c r="A23" s="31" t="s">
@@ -4384,6 +4888,18 @@
       <x:c r="G23" s="33" t="s">
         <x:v>142</x:v>
       </x:c>
+      <x:c r="H23" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I23" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J23" s="56" t="str">
+        <x:v>FR-08</x:v>
+      </x:c>
+      <x:c r="K23" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="27">
       <x:c r="A24" s="31" t="s">
@@ -4407,6 +4923,18 @@
       <x:c r="G24" s="33" t="s">
         <x:v>148</x:v>
       </x:c>
+      <x:c r="H24" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I24" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J24" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K24" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="40.5">
       <x:c r="A25" s="31" t="s">
@@ -4430,6 +4958,18 @@
       <x:c r="G25" s="33" t="s">
         <x:v>154</x:v>
       </x:c>
+      <x:c r="H25" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I25" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J25" s="56" t="str">
+        <x:v>FR-22</x:v>
+      </x:c>
+      <x:c r="K25" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="40.5">
       <x:c r="A26" s="31" t="s">
@@ -4453,6 +4993,18 @@
       <x:c r="G26" s="33" t="s">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="H26" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I26" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J26" s="56" t="str">
+        <x:v>FR-21</x:v>
+      </x:c>
+      <x:c r="K26" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="27">
       <x:c r="A27" s="31" t="s">
@@ -4476,6 +5028,18 @@
       <x:c r="G27" s="33" t="s">
         <x:v>166</x:v>
       </x:c>
+      <x:c r="H27" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I27" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J27" s="56" t="str">
+        <x:v>FR-05; FR-06</x:v>
+      </x:c>
+      <x:c r="K27" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="27">
       <x:c r="A28" s="31" t="s">
@@ -4499,6 +5063,18 @@
       <x:c r="G28" s="33" t="s">
         <x:v>171</x:v>
       </x:c>
+      <x:c r="H28" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I28" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J28" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K28" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="40.5">
       <x:c r="A29" s="31" t="s">
@@ -4522,6 +5098,18 @@
       <x:c r="G29" s="33" t="s">
         <x:v>177</x:v>
       </x:c>
+      <x:c r="H29" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I29" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J29" s="56" t="str">
+        <x:v>FR-05</x:v>
+      </x:c>
+      <x:c r="K29" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="27">
       <x:c r="A30" s="31" t="s">
@@ -4545,6 +5133,18 @@
       <x:c r="G30" s="33" t="s">
         <x:v>183</x:v>
       </x:c>
+      <x:c r="H30" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I30" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J30" s="56" t="str">
+        <x:v>FR-03</x:v>
+      </x:c>
+      <x:c r="K30" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="40.5">
       <x:c r="A31" s="31" t="s">
@@ -4568,6 +5168,18 @@
       <x:c r="G31" s="33" t="s">
         <x:v>189</x:v>
       </x:c>
+      <x:c r="H31" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I31" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J31" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K31" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="40.5">
       <x:c r="A32" s="31" t="s">
@@ -4591,6 +5203,18 @@
       <x:c r="G32" s="33" t="s">
         <x:v>189</x:v>
       </x:c>
+      <x:c r="H32" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I32" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J32" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K32" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="27">
       <x:c r="A33" s="31" t="s">
@@ -4614,6 +5238,18 @@
       <x:c r="G33" s="33" t="s">
         <x:v>189</x:v>
       </x:c>
+      <x:c r="H33" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I33" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J33" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K33" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="31" t="s">
@@ -4637,6 +5273,18 @@
       <x:c r="G34" s="33" t="s">
         <x:v>204</x:v>
       </x:c>
+      <x:c r="H34" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I34" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J34" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K34" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="31" t="s">
@@ -4660,6 +5308,18 @@
       <x:c r="G35" s="33" t="s">
         <x:v>210</x:v>
       </x:c>
+      <x:c r="H35" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I35" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J35" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K35" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="27">
       <x:c r="A36" s="31" t="s">
@@ -4683,6 +5343,18 @@
       <x:c r="G36" s="33" t="s">
         <x:v>216</x:v>
       </x:c>
+      <x:c r="H36" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I36" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J36" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K36" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="31" t="s">
@@ -4706,6 +5378,18 @@
       <x:c r="G37" s="33" t="s">
         <x:v>221</x:v>
       </x:c>
+      <x:c r="H37" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I37" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J37" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K37" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="31" t="s">
@@ -4729,6 +5413,18 @@
       <x:c r="G38" s="33" t="s">
         <x:v>227</x:v>
       </x:c>
+      <x:c r="H38" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I38" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J38" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K38" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="31" t="s">
@@ -4752,6 +5448,18 @@
       <x:c r="G39" s="33" t="s">
         <x:v>233</x:v>
       </x:c>
+      <x:c r="H39" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I39" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J39" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K39" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="27">
       <x:c r="A40" s="31" t="s">
@@ -4775,6 +5483,18 @@
       <x:c r="G40" s="33" t="s">
         <x:v>238</x:v>
       </x:c>
+      <x:c r="H40" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I40" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J40" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K40" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="27">
       <x:c r="A41" s="31" t="s">
@@ -4798,6 +5518,18 @@
       <x:c r="G41" s="33" t="s">
         <x:v>244</x:v>
       </x:c>
+      <x:c r="H41" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I41" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J41" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K41" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="27">
       <x:c r="A42" s="31" t="s">
@@ -4821,6 +5553,18 @@
       <x:c r="G42" s="33" t="s">
         <x:v>248</x:v>
       </x:c>
+      <x:c r="H42" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I42" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J42" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K42" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="31" t="s">
@@ -4844,6 +5588,18 @@
       <x:c r="G43" s="33" t="s">
         <x:v>254</x:v>
       </x:c>
+      <x:c r="H43" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I43" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J43" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K43" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="31" t="s">
@@ -4867,6 +5623,18 @@
       <x:c r="G44" s="33" t="s">
         <x:v>260</x:v>
       </x:c>
+      <x:c r="H44" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I44" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J44" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K44" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="27">
       <x:c r="A45" s="31" t="s">
@@ -4890,6 +5658,18 @@
       <x:c r="G45" s="33" t="s">
         <x:v>265</x:v>
       </x:c>
+      <x:c r="H45" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I45" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J45" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K45" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="31" t="s">
@@ -4913,6 +5693,18 @@
       <x:c r="G46" s="33" t="s">
         <x:v>269</x:v>
       </x:c>
+      <x:c r="H46" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I46" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J46" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K46" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="31" t="s">
@@ -4936,6 +5728,18 @@
       <x:c r="G47" s="33" t="s">
         <x:v>274</x:v>
       </x:c>
+      <x:c r="H47" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I47" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J47" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K47" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="27">
       <x:c r="A48" s="31" t="s">
@@ -4959,6 +5763,18 @@
       <x:c r="G48" s="33" t="s">
         <x:v>280</x:v>
       </x:c>
+      <x:c r="H48" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I48" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J48" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K48" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="27">
       <x:c r="A49" s="31" t="s">
@@ -4982,6 +5798,18 @@
       <x:c r="G49" s="33" t="s">
         <x:v>286</x:v>
       </x:c>
+      <x:c r="H49" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I49" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J49" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K49" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="27">
       <x:c r="A50" s="31" t="s">
@@ -5005,6 +5833,18 @@
       <x:c r="G50" s="33" t="s">
         <x:v>291</x:v>
       </x:c>
+      <x:c r="H50" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I50" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J50" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K50" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="31" t="s">
@@ -5028,6 +5868,18 @@
       <x:c r="G51" s="33" t="s">
         <x:v>297</x:v>
       </x:c>
+      <x:c r="H51" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I51" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J51" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K51" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="31" t="s">
@@ -5051,6 +5903,18 @@
       <x:c r="G52" s="33" t="s">
         <x:v>303</x:v>
       </x:c>
+      <x:c r="H52" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I52" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J52" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K52" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="27">
       <x:c r="A53" s="31" t="s">
@@ -5074,6 +5938,18 @@
       <x:c r="G53" s="33" t="s">
         <x:v>309</x:v>
       </x:c>
+      <x:c r="H53" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I53" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J53" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K53" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="27">
       <x:c r="A54" s="31" t="s">
@@ -5097,6 +5973,18 @@
       <x:c r="G54" s="33" t="s">
         <x:v>315</x:v>
       </x:c>
+      <x:c r="H54" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I54" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J54" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K54" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="27">
       <x:c r="A55" s="31" t="s">
@@ -5120,6 +6008,18 @@
       <x:c r="G55" s="33" t="s">
         <x:v>321</x:v>
       </x:c>
+      <x:c r="H55" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I55" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J55" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K55" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="27">
       <x:c r="A56" s="31" t="s">
@@ -5143,6 +6043,18 @@
       <x:c r="G56" s="33" t="s">
         <x:v>325</x:v>
       </x:c>
+      <x:c r="H56" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I56" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J56" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K56" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="27">
       <x:c r="A57" s="31" t="s">
@@ -5166,6 +6078,18 @@
       <x:c r="G57" s="33" t="s">
         <x:v>330</x:v>
       </x:c>
+      <x:c r="H57" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I57" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J57" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K57" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="27">
       <x:c r="A58" s="31" t="s">
@@ -5189,6 +6113,18 @@
       <x:c r="G58" s="33" t="s">
         <x:v>335</x:v>
       </x:c>
+      <x:c r="H58" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I58" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J58" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K58" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="40.5">
       <x:c r="A59" s="31" t="s">
@@ -5212,6 +6148,18 @@
       <x:c r="G59" s="33" t="s">
         <x:v>339</x:v>
       </x:c>
+      <x:c r="H59" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I59" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J59" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K59" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="40.5">
       <x:c r="A60" s="31" t="s">
@@ -5235,6 +6183,18 @@
       <x:c r="G60" s="33" t="s">
         <x:v>339</x:v>
       </x:c>
+      <x:c r="H60" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I60" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J60" s="56" t="str">
+        <x:v>Supporting NFR reliability/usability; no net-new FR</x:v>
+      </x:c>
+      <x:c r="K60" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="27">
       <x:c r="A61" s="31" t="s">
@@ -5258,6 +6218,18 @@
       <x:c r="G61" s="33" t="s">
         <x:v>348</x:v>
       </x:c>
+      <x:c r="H61" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I61" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J61" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K61" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="31" t="s">
@@ -5281,6 +6253,18 @@
       <x:c r="G62" s="33" t="s">
         <x:v>352</x:v>
       </x:c>
+      <x:c r="H62" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I62" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J62" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K62" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="31" t="s">
@@ -5304,6 +6288,18 @@
       <x:c r="G63" s="33" t="s">
         <x:v>357</x:v>
       </x:c>
+      <x:c r="H63" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I63" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J63" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K63" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="27">
       <x:c r="A64" s="31" t="s">
@@ -5327,6 +6323,18 @@
       <x:c r="G64" s="33" t="s">
         <x:v>362</x:v>
       </x:c>
+      <x:c r="H64" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I64" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J64" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K64" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="31" t="s">
@@ -5350,6 +6358,18 @@
       <x:c r="G65" s="33" t="s">
         <x:v>368</x:v>
       </x:c>
+      <x:c r="H65" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I65" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J65" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K65" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="31" t="s">
@@ -5373,6 +6393,18 @@
       <x:c r="G66" s="33" t="s">
         <x:v>373</x:v>
       </x:c>
+      <x:c r="H66" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I66" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J66" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K66" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="37" t="s">
@@ -5396,6 +6428,18 @@
       <x:c r="G67" s="39" t="s">
         <x:v>378</x:v>
       </x:c>
+      <x:c r="H67" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I67" s="56" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="J67" s="56" t="str">
+        <x:v>Supporting SRS integration and operability</x:v>
+      </x:c>
+      <x:c r="K67" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="27">
       <x:c r="A68" s="41" t="s">
@@ -5419,6 +6463,18 @@
       <x:c r="G68" s="43" t="s">
         <x:v>383</x:v>
       </x:c>
+      <x:c r="H68" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I68" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J68" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K68" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="27">
       <x:c r="A69" s="41" t="s">
@@ -5442,6 +6498,18 @@
       <x:c r="G69" s="43" t="s">
         <x:v>388</x:v>
       </x:c>
+      <x:c r="H69" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I69" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J69" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K69" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="27">
       <x:c r="A70" s="41" t="s">
@@ -5465,6 +6533,18 @@
       <x:c r="G70" s="43" t="s">
         <x:v>394</x:v>
       </x:c>
+      <x:c r="H70" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I70" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J70" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K70" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="27">
       <x:c r="A71" s="41" t="s">
@@ -5488,6 +6568,18 @@
       <x:c r="G71" s="43" t="s">
         <x:v>400</x:v>
       </x:c>
+      <x:c r="H71" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I71" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J71" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K71" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="41" t="s">
@@ -5511,6 +6603,18 @@
       <x:c r="G72" s="43" t="s">
         <x:v>406</x:v>
       </x:c>
+      <x:c r="H72" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I72" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J72" s="56" t="str">
+        <x:v>Supporting usability; SEC-01</x:v>
+      </x:c>
+      <x:c r="K72" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="27">
       <x:c r="A73" s="41" t="s">
@@ -5534,6 +6638,18 @@
       <x:c r="G73" s="43" t="s">
         <x:v>412</x:v>
       </x:c>
+      <x:c r="H73" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I73" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J73" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K73" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="27">
       <x:c r="A74" s="41" t="s">
@@ -5557,6 +6673,18 @@
       <x:c r="G74" s="43" t="s">
         <x:v>417</x:v>
       </x:c>
+      <x:c r="H74" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I74" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J74" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K74" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="27">
       <x:c r="A75" s="41" t="s">
@@ -5580,6 +6708,18 @@
       <x:c r="G75" s="43" t="s">
         <x:v>422</x:v>
       </x:c>
+      <x:c r="H75" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I75" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J75" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K75" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="27">
       <x:c r="A76" s="41" t="s">
@@ -5603,6 +6743,18 @@
       <x:c r="G76" s="43" t="s">
         <x:v>427</x:v>
       </x:c>
+      <x:c r="H76" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I76" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J76" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K76" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="27">
       <x:c r="A77" s="41" t="s">
@@ -5626,6 +6778,18 @@
       <x:c r="G77" s="43" t="s">
         <x:v>433</x:v>
       </x:c>
+      <x:c r="H77" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I77" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J77" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K77" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="40.5">
       <x:c r="A78" s="41" t="s">
@@ -5649,6 +6813,18 @@
       <x:c r="G78" s="43" t="s">
         <x:v>439</x:v>
       </x:c>
+      <x:c r="H78" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I78" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J78" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K78" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="27">
       <x:c r="A79" s="41" t="s">
@@ -5672,6 +6848,18 @@
       <x:c r="G79" s="43" t="s">
         <x:v>444</x:v>
       </x:c>
+      <x:c r="H79" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I79" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J79" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K79" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="27">
       <x:c r="A80" s="41" t="s">
@@ -5695,6 +6883,18 @@
       <x:c r="G80" s="43" t="s">
         <x:v>449</x:v>
       </x:c>
+      <x:c r="H80" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I80" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J80" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K80" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="41" t="s">
@@ -5718,6 +6918,18 @@
       <x:c r="G81" s="43" t="s">
         <x:v>454</x:v>
       </x:c>
+      <x:c r="H81" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I81" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J81" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K81" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="27">
       <x:c r="A82" s="41" t="s">
@@ -5741,6 +6953,18 @@
       <x:c r="G82" s="43" t="s">
         <x:v>460</x:v>
       </x:c>
+      <x:c r="H82" s="56" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="I82" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J82" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K82" s="56" t="str">
+        <x:v>Existing behavior/configuration was present but defective, unsafe, inconsistent, or non-operational; the change restores intended behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="27">
       <x:c r="A83" s="41" t="s">
@@ -5764,6 +6988,18 @@
       <x:c r="G83" s="43" t="s">
         <x:v>465</x:v>
       </x:c>
+      <x:c r="H83" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I83" s="56" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="J83" s="56" t="str">
+        <x:v>SEC-01; SEC-06; FR-01 to FR-04</x:v>
+      </x:c>
+      <x:c r="K83" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="27">
       <x:c r="A84" s="41" t="s">
@@ -5787,6 +7023,18 @@
       <x:c r="G84" s="43" t="s">
         <x:v>471</x:v>
       </x:c>
+      <x:c r="H84" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I84" s="56" t="str">
+        <x:v>Phase 2 — Fabric Identity</x:v>
+      </x:c>
+      <x:c r="J84" s="56" t="str">
+        <x:v>SEC-02; SEC-06; SEC-08; identity-bound FRs</x:v>
+      </x:c>
+      <x:c r="K84" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="27">
       <x:c r="A85" s="41" t="s">
@@ -5810,6 +7058,18 @@
       <x:c r="G85" s="43" t="s">
         <x:v>477</x:v>
       </x:c>
+      <x:c r="H85" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I85" s="56" t="str">
+        <x:v>Phase 2 — Fabric Identity</x:v>
+      </x:c>
+      <x:c r="J85" s="56" t="str">
+        <x:v>SEC-02; SEC-06; SEC-08; identity-bound FRs</x:v>
+      </x:c>
+      <x:c r="K85" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="27">
       <x:c r="A86" s="41" t="s">
@@ -5833,6 +7093,18 @@
       <x:c r="G86" s="43" t="s">
         <x:v>483</x:v>
       </x:c>
+      <x:c r="H86" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I86" s="56" t="str">
+        <x:v>Phase 2 — Fabric Identity</x:v>
+      </x:c>
+      <x:c r="J86" s="56" t="str">
+        <x:v>SEC-02; SEC-06; SEC-08; identity-bound FRs</x:v>
+      </x:c>
+      <x:c r="K86" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="40.5">
       <x:c r="A87" s="41" t="s">
@@ -5856,6 +7128,18 @@
       <x:c r="G87" s="43" t="s">
         <x:v>489</x:v>
       </x:c>
+      <x:c r="H87" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I87" s="56" t="str">
+        <x:v>Phase 2 — Fabric Identity</x:v>
+      </x:c>
+      <x:c r="J87" s="56" t="str">
+        <x:v>SEC-02; SEC-06; SEC-08; identity-bound FRs</x:v>
+      </x:c>
+      <x:c r="K87" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="27">
       <x:c r="A88" s="41" t="s">
@@ -5879,6 +7163,18 @@
       <x:c r="G88" s="43" t="s">
         <x:v>494</x:v>
       </x:c>
+      <x:c r="H88" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I88" s="56" t="str">
+        <x:v>Phase 3 — API Parity</x:v>
+      </x:c>
+      <x:c r="J88" s="56" t="str">
+        <x:v>SRS Section 5; FR-07 to FR-27 as routed</x:v>
+      </x:c>
+      <x:c r="K88" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="27">
       <x:c r="A89" s="41" t="s">
@@ -5902,6 +7198,18 @@
       <x:c r="G89" s="43" t="s">
         <x:v>499</x:v>
       </x:c>
+      <x:c r="H89" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I89" s="56" t="str">
+        <x:v>Phase 3 — API Parity</x:v>
+      </x:c>
+      <x:c r="J89" s="56" t="str">
+        <x:v>SEC-02; SEC-08; FR-10; FR-14</x:v>
+      </x:c>
+      <x:c r="K89" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="27">
       <x:c r="A90" s="41" t="s">
@@ -5925,6 +7233,18 @@
       <x:c r="G90" s="43" t="s">
         <x:v>505</x:v>
       </x:c>
+      <x:c r="H90" s="56" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I90" s="56" t="str">
+        <x:v>Phase 3 — API Parity</x:v>
+      </x:c>
+      <x:c r="J90" s="56" t="str">
+        <x:v>SRS Section 5; FR-07 to FR-27 as routed</x:v>
+      </x:c>
+      <x:c r="K90" s="56" t="str">
+        <x:v>The change repairs an existing broken path and also extends it to participate in the SRS-compliant workflow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="27">
       <x:c r="A91" s="41" t="s">
@@ -5948,6 +7268,18 @@
       <x:c r="G91" s="43" t="s">
         <x:v>511</x:v>
       </x:c>
+      <x:c r="H91" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I91" s="56" t="str">
+        <x:v>Phase 3 — API Parity</x:v>
+      </x:c>
+      <x:c r="J91" s="56" t="str">
+        <x:v>SRS Section 5; FR-07 to FR-27 as routed</x:v>
+      </x:c>
+      <x:c r="K91" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
@@ -5971,6 +7303,18 @@
       <x:c r="G92" t="str">
         <x:v>Completes FR-05 to FR-10 while keeping PII off-chain.</x:v>
       </x:c>
+      <x:c r="H92" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I92" s="56" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="J92" s="56" t="str">
+        <x:v>FR-05 to FR-10; SEC-03</x:v>
+      </x:c>
+      <x:c r="K92" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="str">
@@ -5994,6 +7338,18 @@
       <x:c r="G93" t="str">
         <x:v>Makes MySQL authoritative for detailed patient PII and clinical/admin data.</x:v>
       </x:c>
+      <x:c r="H93" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I93" s="56" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="J93" s="56" t="str">
+        <x:v>FR-05 to FR-10; SEC-03</x:v>
+      </x:c>
+      <x:c r="K93" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="str">
@@ -6017,6 +7373,18 @@
       <x:c r="G94" t="str">
         <x:v>Aligns new patient writes with SEC-03; historical ledger PII cleanup remains a deployment gate.</x:v>
       </x:c>
+      <x:c r="H94" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I94" s="56" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="J94" s="56" t="str">
+        <x:v>SEC-03; FR-05 to FR-10</x:v>
+      </x:c>
+      <x:c r="K94" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="str">
@@ -6040,6 +7408,18 @@
       <x:c r="G95" t="str">
         <x:v>Preserves Phase 1 JWT and Phase 2 MSP/RBAC binding.</x:v>
       </x:c>
+      <x:c r="H95" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I95" s="56" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="J95" s="56" t="str">
+        <x:v>SEC-03; FR-05 to FR-10</x:v>
+      </x:c>
+      <x:c r="K95" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
@@ -6063,6 +7443,18 @@
       <x:c r="G96" t="str">
         <x:v>Completes admin patient-management workflow.</x:v>
       </x:c>
+      <x:c r="H96" s="56" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I96" s="56" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="J96" s="56" t="str">
+        <x:v>FR-05 to FR-10; SEC-03</x:v>
+      </x:c>
+      <x:c r="K96" s="56" t="str">
+        <x:v>The baseline lacked a required SRS capability or security control; the change adds new product behavior or enforcement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="str">
@@ -6085,6 +7477,18 @@
       </x:c>
       <x:c r="G97" t="str">
         <x:v>Protects API coverage and SEC-03 design.</x:v>
+      </x:c>
+      <x:c r="H97" s="56" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I97" s="56" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="J97" s="56" t="str">
+        <x:v>FR-05 to FR-10; SEC-03</x:v>
+      </x:c>
+      <x:c r="K97" s="56" t="str">
+        <x:v>This entry supplies tests, documentation, migration, or deployment evidence and does not independently add end-user behavior.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6125,7 +7529,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7041ad5563334f85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86d733fd0ac443d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6315,7 +7719,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5db5c180376429a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd251c6124c664d9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6689,7 +8093,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bf2a89aaf62490c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bff09c5ec734593"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6802,7 +8206,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44441e59a084a43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref3e871e15284c54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6957,7 +8361,7 @@
         <x:v>Back up MySQL; apply migration; DESCRIBE Patient; verify unique Emirates_ID and clinic FK/index.</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Pending AWS deployment.</x:v>
+        <x:v>Passed 2026-07-11. edr_db backed up; clinics 1/2 seeded; ten Phase 4 columns, both indexes, and fk_patient_clinic verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6977,7 +8381,7 @@
         <x:v>Package/install/approve/commit next basic version and sequence; sanitize historical patient state containing PII.</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>Pending AWS deployment.</x:v>
+        <x:v>Passed 2026-07-11. Chaincode basic 1.0.3 sequence 5 committed with Org1MSP and Org2MSP approvals; Patient1-Patient3 sanitized.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6997,7 +8401,7 @@
         <x:v>Restart both PM2 APIs; clean-install/build frontend; copy dist to /var/www/edr; run authenticated create/update/read/assign/delete and negative role/clinic/owner smoke tests.</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>Pending AWS deployment.</x:v>
+        <x:v>Deployed 2026-07-11. APIs restarted, frontend rebuilt/copied to Nginx, and full create/update/read/assign/owner/delete smoke flow passed. Final delete-row fix commit 6d48146 awaits pull/rebuild; two legacy ledger-only patients await preservation/sanitization.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7257,16 +8661,20 @@
         <x:v>FR-05 to FR-10</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>Source complete</x:v>
+        <x:v>Deployed with final delete-row correction pending</x:v>
       </x:c>
       <x:c r="D11" t="str">
         <x:v>Hybrid patient CRUD/assignment with all SRS fields, UUID and UI actions.</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>AWS deploy and smoke validation pending.</x:v>
-      </x:c>
-      <x:c r="F11" t="str"/>
-      <x:c r="G11" t="str"/>
+        <x:v>FR-05 to FR-10</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Full AWS workflow passed; commit 6d48146 fixes explicit Patient subtype deletion.</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Pull/rebuild 6d48146 and rerun cleanup verification.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
@@ -7276,18 +8684,361 @@
         <x:v>SEC-03</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Source complete for new patient writes</x:v>
+        <x:v>Deployed for mapped patients</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>MySQL PII plus Fabric reference/SHA-256 metadata only.</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>Historical patient ledger PII cleanup and Phase 5 doctor split pending.</x:v>
-      </x:c>
-      <x:c r="F12" t="str"/>
-      <x:c r="G12" t="str"/>
+        <x:v>SEC-03</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Patient1-Patient3 sanitized; chaincode 1.0.3 sequence 5 committed.</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Preserve/import and sanitize ledger-only Patient5 and PatientQA001; Phase 5 handles doctor PII.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="105" t="str">
+        <x:v>Remediation Classification Summary — Phases 1 to 4</x:v>
+      </x:c>
+      <x:c r="B1" s="105"/>
+      <x:c r="C1" s="105"/>
+      <x:c r="D1" s="105"/>
+      <x:c r="E1" s="105"/>
+      <x:c r="F1" s="105"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="106" t="str">
+        <x:v>Evidence-based distinction between corrections to existing behavior and development performed to close SRS gaps.</x:v>
+      </x:c>
+      <x:c r="B2" s="106"/>
+      <x:c r="C2" s="106"/>
+      <x:c r="D2" s="106"/>
+      <x:c r="E2" s="106"/>
+      <x:c r="F2" s="106"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="56"/>
+      <x:c r="B3" s="56"/>
+      <x:c r="C3" s="56"/>
+      <x:c r="D3" s="56"/>
+      <x:c r="E3" s="56"/>
+      <x:c r="F3" s="56"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="107" t="str">
+        <x:v>Work Type</x:v>
+      </x:c>
+      <x:c r="B4" s="107" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="C4" s="107" t="str">
+        <x:v>Definition</x:v>
+      </x:c>
+      <x:c r="D4" s="56"/>
+      <x:c r="E4" s="56"/>
+      <x:c r="F4" s="56"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="84" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$97,A5)</x:f>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C5" s="86" t="str">
+        <x:v>Corrects behavior/configuration that existed but was defective, unsafe, inconsistent, or non-operational.</x:v>
+      </x:c>
+      <x:c r="D5" s="56"/>
+      <x:c r="E5" s="56"/>
+      <x:c r="F5" s="56"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="87" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="B6" s="88" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$97,A6)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C6" s="89" t="str">
+        <x:v>Adds a required SRS capability or security control that did not exist in the baseline.</x:v>
+      </x:c>
+      <x:c r="D6" s="56"/>
+      <x:c r="E6" s="56"/>
+      <x:c r="F6" s="56"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="87" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="B7" s="88" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$97,A7)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C7" s="89" t="str">
+        <x:v>Repairs an existing path while materially extending it for an SRS-compliant workflow.</x:v>
+      </x:c>
+      <x:c r="D7" s="56"/>
+      <x:c r="E7" s="56"/>
+      <x:c r="F7" s="56"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="90" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="B8" s="91" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$97,A8)</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C8" s="92" t="str">
+        <x:v>Tests, documentation, migrations, or deployment evidence; not independently end-user functionality.</x:v>
+      </x:c>
+      <x:c r="D8" s="56"/>
+      <x:c r="E8" s="56"/>
+      <x:c r="F8" s="56"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="56"/>
+      <x:c r="B9" s="56"/>
+      <x:c r="C9" s="56"/>
+      <x:c r="D9" s="56"/>
+      <x:c r="E9" s="56"/>
+      <x:c r="F9" s="56"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="107" t="str">
+        <x:v>Phase</x:v>
+      </x:c>
+      <x:c r="B10" s="107" t="str">
+        <x:v>Bug Fix</x:v>
+      </x:c>
+      <x:c r="C10" s="107" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="D10" s="107" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="E10" s="107" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="F10" s="107" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="84" t="str">
+        <x:v>Baseline Stabilization</x:v>
+      </x:c>
+      <x:c r="B11" s="85" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A11,'Changes'!$H$2:$H$97,B$10)</x:f>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C11" s="85" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A11,'Changes'!$H$2:$H$97,C$10)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D11" s="85" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A11,'Changes'!$H$2:$H$97,D$10)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E11" s="85" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A11,'Changes'!$H$2:$H$97,E$10)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="n">
+        <x:f>SUM(B11:E11)</x:f>
+        <x:v>66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="87" t="str">
+        <x:v>Phase 1 — API Authentication</x:v>
+      </x:c>
+      <x:c r="B12" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A12,'Changes'!$H$2:$H$97,B$10)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C12" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A12,'Changes'!$H$2:$H$97,C$10)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D12" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A12,'Changes'!$H$2:$H$97,D$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A12,'Changes'!$H$2:$H$97,E$10)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F12" s="94" t="n">
+        <x:f>SUM(B12:E12)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="87" t="str">
+        <x:v>Phase 2 — Fabric Identity</x:v>
+      </x:c>
+      <x:c r="B13" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A13,'Changes'!$H$2:$H$97,B$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A13,'Changes'!$H$2:$H$97,C$10)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D13" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A13,'Changes'!$H$2:$H$97,D$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A13,'Changes'!$H$2:$H$97,E$10)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F13" s="94" t="n">
+        <x:f>SUM(B13:E13)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="87" t="str">
+        <x:v>Phase 3 — API Parity</x:v>
+      </x:c>
+      <x:c r="B14" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A14,'Changes'!$H$2:$H$97,B$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A14,'Changes'!$H$2:$H$97,C$10)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D14" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A14,'Changes'!$H$2:$H$97,D$10)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="88" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A14,'Changes'!$H$2:$H$97,E$10)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F14" s="94" t="n">
+        <x:f>SUM(B14:E14)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="90" t="str">
+        <x:v>Phase 4 — Patient Management</x:v>
+      </x:c>
+      <x:c r="B15" s="91" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A15,'Changes'!$H$2:$H$97,B$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="91" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A15,'Changes'!$H$2:$H$97,C$10)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D15" s="91" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A15,'Changes'!$H$2:$H$97,D$10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="91" t="n">
+        <x:f>COUNTIFS('Changes'!$I$2:$I$97,$A15,'Changes'!$H$2:$H$97,E$10)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F15" s="95" t="n">
+        <x:f>SUM(B15:E15)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="56"/>
+      <x:c r="B16" s="56"/>
+      <x:c r="C16" s="56"/>
+      <x:c r="D16" s="56"/>
+      <x:c r="E16" s="56"/>
+      <x:c r="F16" s="56"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="107" t="str">
+        <x:v>Interpretation Notes</x:v>
+      </x:c>
+      <x:c r="B17" s="107"/>
+      <x:c r="C17" s="107"/>
+      <x:c r="D17" s="107"/>
+      <x:c r="E17" s="107"/>
+      <x:c r="F17" s="107"/>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="56" t="str">
+        <x:v>1. Classification is based on baseline behavior and SRS obligation, not the filename or engineering discipline.</x:v>
+      </x:c>
+      <x:c r="B18" s="56"/>
+      <x:c r="C18" s="56"/>
+      <x:c r="D18" s="56"/>
+      <x:c r="E18" s="56"/>
+      <x:c r="F18" s="56"/>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="56" t="str">
+        <x:v>2. Security controls absent from the baseline are SRS gap development even when they also remediate a vulnerability.</x:v>
+      </x:c>
+      <x:c r="B19" s="56"/>
+      <x:c r="C19" s="56"/>
+      <x:c r="D19" s="56"/>
+      <x:c r="E19" s="56"/>
+      <x:c r="F19" s="56"/>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="56" t="str">
+        <x:v>3. Runtime corrections such as wrong ports, crashes, bad type handling, and incompatible Docker/Fabric settings are bug fixes.</x:v>
+      </x:c>
+      <x:c r="B20" s="56"/>
+      <x:c r="C20" s="56"/>
+      <x:c r="D20" s="56"/>
+      <x:c r="E20" s="56"/>
+      <x:c r="F20" s="56"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="56" t="str">
+        <x:v>4. Documentation and tests are tracked separately so they do not inflate either product-development or defect-remediation totals.</x:v>
+      </x:c>
+      <x:c r="B21" s="56"/>
+      <x:c r="C21" s="56"/>
+      <x:c r="D21" s="56"/>
+      <x:c r="E21" s="56"/>
+      <x:c r="F21" s="56"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A17:F17"/>
+    <x:mergeCell ref="A18:F18"/>
+    <x:mergeCell ref="A19:F19"/>
+    <x:mergeCell ref="A20:F20"/>
+    <x:mergeCell ref="A21:F21"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Phase 9 deployment evidence
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb8914b3e6d85496a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R84241f8a7f8445ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R550071bb746a4286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Raa57b544cfdb48ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="Rddfff5d226194ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R9ca280becc714357"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R105b042f0905400f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="R97c85caf94f444f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf5f0f3fa94834eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R3828c517bf284a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R3fbf152e8c454b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Re6578b13fe444eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R35e01dbbbdbe4b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R931d1d728ea544c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R97d6f5c8e1094a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="Rcfc109e3313e454f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3741,9 +3741,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Complete</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Remediation Classification Summary — Through Phase 7A</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Evidence-based distinction between corrections to existing behavior and development performed to close SRS gaps.</x:t>
@@ -5034,7 +5031,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfd9408a320d04c0f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7559b8a80b3b4af2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5350,8 +5347,8 @@
       <x:c r="B6" s="54" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C6" s="55">
-        <x:v>46215</x:v>
+      <x:c r="C6" s="55" t="str">
+        <x:v>7/15/26</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5393,7 +5390,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="C13" s="60" t="n">
-        <x:v>71</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -5441,7 +5438,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C19" s="65" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -5449,7 +5446,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="C20" s="65" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -5457,7 +5454,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="C21" s="70" t="n">
-        <x:v>142</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="17.25">
@@ -5471,8 +5468,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="C23" s="60" t="n">
-        <x:f>COUNTA(RuntimeTable[ID])</x:f>
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -5480,7 +5476,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="C24" s="60" t="n">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -5488,8 +5484,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C25" s="65" t="n">
-        <x:f>COUNTA('Known Items'!A2:A14)</x:f>
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5499,7 +5494,7 @@
     <x:mergeCell ref="B9:I9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4c2db616f544f3c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4202d643c0ab42b1"/>
 </x:worksheet>
 </file>
 
@@ -10524,6 +10519,146 @@
       </x:c>
       <x:c r="K143" t="str">
         <x:v>Completed deployment closeout only; no planned-only items were added to the workbook.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>P9-01</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>database/migrations/2026-07-15-phase9-appointment-management.sql</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>Persisted appointment lifecycle schema</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>The legacy table lacked generated IDs, time-of-day, specialty, status, cancellation, and modification evidence.</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>Added and deployed the Phase 9 migration with safe legacy backfill and schema verification.</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>Supports durable create/update/cancel and upcoming/past history.</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I144" t="str">
+        <x:v>Phase 9 - Appointment Management</x:v>
+      </x:c>
+      <x:c r="J144" t="str">
+        <x:v>FR-29; FR-30; FR-31</x:v>
+      </x:c>
+      <x:c r="K144" t="str">
+        <x:v>Applied on AWS 2026-07-15; backup contains pre-migration MySQL dump.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>P9-02</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>backend/server.js; dental-backend/test/phase9AppointmentManagement.test.js</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>Scoped appointment APIs</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>Appointment creation/update/cancellation were absent and the legacy read route was read-only.</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>Added JWT role/clinic/patient scoped list, create, update, cancel, and appointment-doctor option APIs with focused tests.</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>Admin appointment lifecycle and patient-owned history are enforced server-side.</x:v>
+      </x:c>
+      <x:c r="H145" t="str">
+        <x:v>SRS Gap Development</x:v>
+      </x:c>
+      <x:c r="I145" t="str">
+        <x:v>Phase 9 - Appointment Management</x:v>
+      </x:c>
+      <x:c r="J145" t="str">
+        <x:v>FR-29; FR-30; FR-31; FR-03</x:v>
+      </x:c>
+      <x:c r="K145" t="str">
+        <x:v>Legacy null-clinic doctors require an existing assignment to the patient; no clinic value is inferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>P9-03</x:v>
+      </x:c>
+      <x:c r="B146" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>bc-dentistry-frontend; BC-Dentistry-Mobile-App</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>Persisted web and authenticated mobile appointment flows</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>Web creation and ticket actions were static; mobile rendered bundled sample appointments.</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>Connected web create/update/cancel to APIs and mobile upcoming/past retrieval to the JWT patient, grouped by specialty/date.</x:v>
+      </x:c>
+      <x:c r="G146" t="str">
+        <x:v>Replaces false/static appointment behavior with persisted scoped data.</x:v>
+      </x:c>
+      <x:c r="H146" t="str">
+        <x:v>Mixed Remediation</x:v>
+      </x:c>
+      <x:c r="I146" t="str">
+        <x:v>Phase 9 - Appointment Management</x:v>
+      </x:c>
+      <x:c r="J146" t="str">
+        <x:v>FR-29; FR-30; FR-31; FR-03</x:v>
+      </x:c>
+      <x:c r="K146" t="str">
+        <x:v>Mobile source/API verified; packaged-device screenshots remain a later evidence gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>P9-04</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>Tests / Deployment</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>AWS /home/ubuntu/EDR; /var/www/edr; database migration; Phase 9 smoke</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>Phase 9 deployment and authenticated runtime evidence</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>Source completion required migration, Git alignment, service rollout, and role/scope smoke evidence.</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>Aligned VM Git to f3f8526, applied migration, rebuilt API/frontend, reloaded Nginx, and passed authenticated create/update/cancel/upcoming/past/denial smoke.</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>Closes the Phase 9 runtime gate.</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I147" t="str">
+        <x:v>Phase 9 - Appointment Management</x:v>
+      </x:c>
+      <x:c r="J147" t="str">
+        <x:v>FR-29; FR-30; FR-31; SRS Section 8</x:v>
+      </x:c>
+      <x:c r="K147" t="str">
+        <x:v>Backup /home/ubuntu/deployment-backups/20260715-085512-phase9-predeploy; marker PHASE9_APPOINTMENT_SMOKE_OK.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10555,7 +10690,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fd2db29390d42cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c9d78e2894b4409"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10742,10 +10877,44 @@
         <x:v>908</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>R-10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>.deployment/phase9-deploy.sh; phase9-followup-deploy.sh; phase9-smoke.js</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Deployment and smoke scripts</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Created for Git alignment, backup, migration, API/frontend rollout, and authenticated appointment verification.</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Reproducible Phase 9 AWS evidence without embedded credentials.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>R-11</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>/home/ubuntu/deployment-backups/20260715-085512-phase9-predeploy</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>AWS deployment backup</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Captured pre-alignment Git state, tracked payload, frontend, and MySQL dump.</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Rollback evidence for Phase 9 deployment.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra52b57b8002d41a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03e1ac080a484cc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11354,6 +11523,39 @@
         <x:v>Pass</x:v>
       </x:c>
     </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>Phase 9 source regression suites</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>Pass. Backend/API syntax and 33/33 tests passed; frontend/mobile integration source tests 8/8 passed.</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>Phase 9 AWS build and migration gates</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>Pass with inherited warnings. VM checkout f3f8526; migration applied and schema inspected; Database API rebuilt; frontend lint/build passed; Nginx validated/reloaded.</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>Pass (warnings)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>Phase 9 authenticated appointment smoke</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>Pass. Admin create/update/cancel, patient upcoming/past/cancelled history, and patient mutation denial passed; marker PHASE9_APPOINTMENT_SMOKE_OK.</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C2:C47">
     <x:cfRule type="expression" dxfId="10" priority="1">
@@ -11368,7 +11570,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40325519e5f641f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0ea35358784dca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11490,10 +11692,26 @@
       <x:c r="A14"/>
       <x:c r="B14"/>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>Phase 9 legacy doctor clinic linkage</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Existing doctors have null Clinic_ID pending authoritative data. Appointment selection permits them only through an existing assignment to a patient in the authenticated admin clinic; no clinic is inferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>Phase 9 packaged mobile evidence</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Authenticated mobile source/API behavior is verified; packaged iOS/Android runtime screenshots and device interaction evidence remain for Phase 10/12.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78c0078050304e61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f0af3a94f8047f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11931,6 +12149,46 @@
         <x:v>Passed 2026-07-14. Initial `basic` 1.0.8 sequence 10 was superseded after Fabric JavaScript default-parameter metadata arity mismatch; final `basic` 1.0.9 sequence 11 committed with Org1MSP/Org2MSP approvals and smoke marker `PHASE8_CONSENT_AUDIT_SMOKE_OK`.</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>P9-DB-01</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Appointment lifecycle database migration</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Yes, before Phase 9 Database API restart</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>database/migrations/2026-07-15-phase9-appointment-management.sql</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Back up MySQL; apply migration; verify Appointment columns; rebuild Database API.</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Passed 2026-07-15. Auto-increment, datetime, specialty, status, cancellation, and modified columns verified on AWS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>P9-APP-01</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Appointment API/web rollout and smoke</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Yes, after database migration</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>backend; bc-dentistry-frontend; Phase 9 deployment/smoke scripts</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Align Git, rebuild Database API/frontend, copy to Nginx, run authenticated appointment smoke.</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>Passed 2026-07-15 at f3f8526. No Fabric upgrade; basic remains 1.0.9 sequence 11.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12338,6 +12596,29 @@
         <x:v>External push notification delivery and packaged mobile-device runtime evidence remain separate if required; the deployed implementation covers in-app ledger notifications and API/web consent workflow.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>P9-FR29-31</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Appointment lifecycle and patient history</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>The SRS requires admin create/update/cancel and patient upcoming/past views organized by specialty/date.</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Only a scoped legacy read existed; web/mobile mutations and mobile history were static or absent.</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>FR-29; FR-30; FR-31; FR-03</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Deployed at f3f8526. Migration, API/UI/mobile source, 33/33 API tests, 8/8 frontend tests, and authenticated AWS smoke passed.</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Packaged mobile-device evidence remains; legacy doctor clinic IDs remain null and use assignment-only fallback.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12354,8 +12635,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="2" ht="21">
-      <x:c r="B2" s="84" t="s">
-        <x:v>1242</x:v>
+      <x:c r="B2" s="84" t="str">
+        <x:v>Remediation Classification Summary — Through Phase 9</x:v>
       </x:c>
       <x:c r="C2" s="84"/>
       <x:c r="D2" s="84"/>
@@ -12365,7 +12646,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="B3" s="85" t="s">
-        <x:v>1243</x:v>
+        <x:v>1242</x:v>
       </x:c>
       <x:c r="C3" s="85"/>
       <x:c r="D3" s="85"/>
@@ -12389,7 +12670,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D5" s="26" t="s">
-        <x:v>1244</x:v>
+        <x:v>1243</x:v>
       </x:c>
       <x:c r="E5" s="13"/>
       <x:c r="F5" s="13"/>
@@ -12399,11 +12680,11 @@
       <x:c r="B6" s="14" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C6" s="20">
-        <x:v>52</x:v>
+      <x:c r="C6" s="20" t="n">
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D6" s="15" t="s">
-        <x:v>1245</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="E6" s="13"/>
       <x:c r="F6" s="13"/>
@@ -12413,11 +12694,11 @@
       <x:c r="B7" s="16" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="C7" s="21">
-        <x:v>43</x:v>
+      <x:c r="C7" s="21" t="n">
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D7" s="17" t="s">
-        <x:v>1246</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="E7" s="13"/>
       <x:c r="F7" s="13"/>
@@ -12427,11 +12708,11 @@
       <x:c r="B8" s="16" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="C8" s="21">
-        <x:v>15</x:v>
+      <x:c r="C8" s="21" t="n">
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D8" s="17" t="s">
-        <x:v>1247</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="E8" s="13"/>
       <x:c r="F8" s="13"/>
@@ -12441,11 +12722,11 @@
       <x:c r="B9" s="18" t="s">
         <x:v>346</x:v>
       </x:c>
-      <x:c r="C9" s="22">
-        <x:v>23</x:v>
+      <x:c r="C9" s="22" t="n">
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D9" s="19" t="s">
-        <x:v>1248</x:v>
+        <x:v>1247</x:v>
       </x:c>
       <x:c r="E9" s="13"/>
       <x:c r="F9" s="13"/>
@@ -12461,7 +12742,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="B11" s="26" t="s">
-        <x:v>1249</x:v>
+        <x:v>1248</x:v>
       </x:c>
       <x:c r="C11" s="26" t="s">
         <x:v>40</x:v>
@@ -12476,7 +12757,7 @@
         <x:v>346</x:v>
       </x:c>
       <x:c r="G11" s="26" t="s">
-        <x:v>1250</x:v>
+        <x:v>1249</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -12695,16 +12976,28 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="B21" s="13"/>
-      <x:c r="C21" s="74"/>
-      <x:c r="D21" s="74"/>
-      <x:c r="E21" s="74"/>
-      <x:c r="F21" s="74"/>
-      <x:c r="G21" s="74"/>
+      <x:c r="B21" s="13" t="str">
+        <x:v>Phases 8–9 — Consent/Audit and Appointments</x:v>
+      </x:c>
+      <x:c r="C21" s="74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="74" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E21" s="74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F21" s="74" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G21" s="74" t="n">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="21">
       <x:c r="B22" s="86" t="s">
-        <x:v>1251</x:v>
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="C22" s="86"/>
       <x:c r="D22" s="86"/>
@@ -12714,7 +13007,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="B23" s="83" t="s">
-        <x:v>1252</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="C23" s="83"/>
       <x:c r="D23" s="83"/>
@@ -12724,7 +13017,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="B24" s="83" t="s">
-        <x:v>1253</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="C24" s="83"/>
       <x:c r="D24" s="83"/>
@@ -12734,7 +13027,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="B25" s="79" t="s">
-        <x:v>1254</x:v>
+        <x:v>1253</x:v>
       </x:c>
       <x:c r="C25" s="79"/>
       <x:c r="D25" s="79"/>
@@ -12744,7 +13037,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="B26" s="79" t="s">
-        <x:v>1255</x:v>
+        <x:v>1254</x:v>
       </x:c>
       <x:c r="C26" s="79"/>
       <x:c r="D26" s="79"/>

</xml_diff>

<commit_message>
fix: preserve clinic key foreign references
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R92f48d81fa184453"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="Rff4a86780e804780"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R2edeec1d55fe493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="R32295937e1dc439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R29c80843490a49ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="Rd0061e8b72ff45a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R3693cc2477004236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="R1579f25cb0504bd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcd136f152be64f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R64826a2e0bac4d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R26083a0c20a2460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rd28f106470ae4f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R4777df77acc84885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R9b09290f05214692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R581f48c00ae34864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="R5f3e64cb7f494d7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6438,7 +6438,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R889b3d3a99be489f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re28fea285ec041bf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -6901,7 +6901,7 @@
     <x:mergeCell ref="B9:I9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d2ca4fbb69f4a48"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ddd76824a3e44e9"/>
 </x:worksheet>
 </file>
 
@@ -12712,10 +12712,10 @@
         <x:v>Clinic lifecycle and mandatory password schema</x:v>
       </x:c>
       <x:c r="E166" t="str">
-        <x:v>Organization identifiers were not auto-generated, clinic status was unavailable, and users had no first-login password-change state.</x:v>
+        <x:v>Clinic status was unavailable, users had no first-login password-change state, and the existing Organization key is referenced by patient foreign keys.</x:v>
       </x:c>
       <x:c r="F166" t="str">
-        <x:v>Adds Organization auto-increment/IsActive and User.Must_Change_Password while preserving Admin.Organization_ID as the primary key.</x:v>
+        <x:v>Adds Organization.IsActive and User.Must_Change_Password while preserving the existing non-auto-increment Organization_ID and Admin.Organization_ID primary key. Clinic creation allocates the next ID inside its transaction.</x:v>
       </x:c>
       <x:c r="G166" t="str">
         <x:v>Supports clinic lifecycle and enforces exactly one Clinic Admin per clinic at the schema boundary.</x:v>
@@ -12902,7 +12902,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2b0d6d395504690"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de3d0c6712f4ce4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13279,7 +13279,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f9d3da80ff74a05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc225d257014447aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14155,7 +14155,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c2fd48088a46f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re730c191307c410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14332,7 +14332,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f0043a754314b45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re41453cfc0e6462a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14984,10 +14984,10 @@
         <x:v>database/migrations/2026-07-21-super-admin-clinic-management.sql</x:v>
       </x:c>
       <x:c r="E32" t="str">
-        <x:v>Back up MySQL; apply migration; verify Organization auto-increment/IsActive, User.Must_Change_Password, and unchanged one-admin-per-clinic Admin primary key.</x:v>
+        <x:v>Back up MySQL; apply migration; verify Organization.IsActive, User.Must_Change_Password, unchanged Organization_ID type, and unchanged one-admin-per-clinic Admin primary key.</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>Source complete; deployment pending.</x:v>
+        <x:v>Source corrected after the first deployment attempt exposed the patient foreign-key dependency; migration and deployment remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">

</xml_diff>

<commit_message>
docs: record clinic governance deployment evidence
</commit_message>
<xml_diff>
--- a/outputs/EDR_fixes.xlsx
+++ b/outputs/EDR_fixes.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcd136f152be64f46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R64826a2e0bac4d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R26083a0c20a2460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rd28f106470ae4f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="R4777df77acc84885"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R9b09290f05214692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="R581f48c00ae34864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="R5f3e64cb7f494d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra7a01397be2d469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" r:id="R342136c8a5d54d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Artifacts" sheetId="3" r:id="R19df146c73744f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="4" r:id="Rf51c91d4e8c94dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Items" sheetId="5" r:id="Rffe5269158ad41a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Migrations" sheetId="6" r:id="R5a2132ac4858411c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SRS Gap Mapping" sheetId="7" r:id="Rd7e262d489cf481e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification Summary" sheetId="8" r:id="R1cb18491d1c44c0f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6438,7 +6438,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re28fea285ec041bf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f389af0ef1f4063"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -6768,7 +6768,7 @@
     </x:row>
     <x:row r="9" ht="33.75" customHeight="1">
       <x:c r="B9" s="83" t="str">
-        <x:v>Scope: completed fixes and source evidence now include Phase 14 application clinic governance. Deployment migration, live role/isolation checks, and clinic-bound Fabric wallet enrollment remain explicit pending items.</x:v>
+        <x:v>Scope: completed fixes and deployment evidence now include the Phase 14 application clinic-governance migration, services, tests, health gates, and authentication guard. Initial Sys Admin bootstrap, authenticated workflow proof, and clinic-bound Fabric wallet enrollment remain explicit pending items.</x:v>
       </x:c>
       <x:c r="C9" s="84"/>
       <x:c r="D9" s="84"/>
@@ -6797,6 +6797,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C13" s="60" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B13)</x:f>
         <x:v>83</x:v>
       </x:c>
     </x:row>
@@ -6805,6 +6806,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="C14" s="60" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B14)</x:f>
         <x:v>19</x:v>
       </x:c>
     </x:row>
@@ -6813,6 +6815,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="C15" s="60" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B15)</x:f>
         <x:v>15</x:v>
       </x:c>
     </x:row>
@@ -6821,6 +6824,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="C16" s="60" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B16)</x:f>
         <x:v>19</x:v>
       </x:c>
     </x:row>
@@ -6829,6 +6833,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="C17" s="65" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B17)</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -6837,6 +6842,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C18" s="65" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B18)</x:f>
         <x:v>9</x:v>
       </x:c>
     </x:row>
@@ -6845,7 +6851,8 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C19" s="65" t="n">
-        <x:v>18</x:v>
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B19)</x:f>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6853,6 +6860,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C20" s="65" t="n">
+        <x:f>COUNTIF('Changes'!$B$2:$B$400,B20)</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -6861,7 +6869,8 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="C21" s="70" t="n">
-        <x:v>169</x:v>
+        <x:f>COUNTA('Changes'!$A$2:$A$400)</x:f>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="17.25">
@@ -6875,7 +6884,8 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C23" s="60" t="n">
-        <x:v>20</x:v>
+        <x:f>COUNTA('Runtime Artifacts'!$A$2:$A$100)</x:f>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6883,7 +6893,8 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="C24" s="60" t="n">
-        <x:v>76</x:v>
+        <x:f>COUNTA('Verification'!$A$2:$A$200)</x:f>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6891,6 +6902,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="C25" s="65" t="n">
+        <x:f>COUNTA('Known Items'!$A$2:$A$100)</x:f>
         <x:v>16</x:v>
       </x:c>
     </x:row>
@@ -6901,7 +6913,7 @@
     <x:mergeCell ref="B9:I9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ddd76824a3e44e9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4368d381d81047fe"/>
 </x:worksheet>
 </file>
 
@@ -12695,7 +12707,7 @@
         <x:v>FR-01; FR-03; multi-clinic onboarding; SEC-01</x:v>
       </x:c>
       <x:c r="K165" t="str">
-        <x:v>Source complete; database deployment and authenticated runtime verification remain pending.</x:v>
+        <x:v>Deployed from commit de9c7ea on 2026-07-21. Database/API/frontend infrastructure is live; initial Sys Admin bootstrap and authenticated clinic workflow evidence remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
@@ -12730,7 +12742,7 @@
         <x:v>FR-01; FR-03; SEC-01; account lifecycle</x:v>
       </x:c>
       <x:c r="K166" t="str">
-        <x:v>Migration authored and reference dump synchronized; not yet applied to the deployment database.</x:v>
+        <x:v>Migration applied on 2026-07-21. Organization.IsActive and User.Must_Change_Password were verified while the existing Organization_ID type and Admin.Organization_ID primary key remained unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -12765,7 +12777,7 @@
         <x:v>FR-01; FR-02; FR-03; SEC-01; SEC-05</x:v>
       </x:c>
       <x:c r="K167" t="str">
-        <x:v>Source complete; initial account creation and first-login runtime proof remain pending.</x:v>
+        <x:v>Bootstrap command and first-login enforcement are deployed. Initial Sys Admin creation and live password-replacement proof await the authorized account email.</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
@@ -12800,7 +12812,7 @@
         <x:v>FR-01; FR-03; role-specific UI; multi-clinic onboarding</x:v>
       </x:c>
       <x:c r="K168" t="str">
-        <x:v>Source complete; live browser and deployed API/database verification remain pending.</x:v>
+        <x:v>Frontend deployed and public route returned HTTP 200. Authenticated Sys Admin browser workflow remains pending until the initial account is bootstrapped.</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -12871,6 +12883,41 @@
       </x:c>
       <x:c r="K170" t="str">
         <x:v>Completed source documentation; deployment/runtime rows remain explicitly pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>P14-DEPLOY-01</x:v>
+      </x:c>
+      <x:c r="B171" t="str">
+        <x:v>Tests / Deployment</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>AWS VM /home/ubuntu/EDR; database/migrations/2026-07-21-super-admin-clinic-management.sql</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>Phase 14 targeted deployment and runtime gates</x:v>
+      </x:c>
+      <x:c r="E171" t="str">
+        <x:v>Phase 14 source and migration had not been applied to the deployment environment.</x:v>
+      </x:c>
+      <x:c r="F171" t="str">
+        <x:v>Backed up the VM and MySQL database, applied the corrected migration, deployed the exact de9c7ea backend/frontend payload, rebuilt only database-api and web-frontend, and verified schema, tests, container health, public endpoints, and the unauthenticated clinic guard.</x:v>
+      </x:c>
+      <x:c r="G171" t="str">
+        <x:v>Provides live deployment evidence without disturbing the dirty VM checkout or representing the unbootstrapped privileged workflow as complete.</x:v>
+      </x:c>
+      <x:c r="H171" t="str">
+        <x:v>Supporting Evidence / Deployment</x:v>
+      </x:c>
+      <x:c r="I171" t="str">
+        <x:v>Phase 14 - Application Clinic Governance</x:v>
+      </x:c>
+      <x:c r="J171" t="str">
+        <x:v>SRS Section 8; deployment; SEC-01; FR-03</x:v>
+      </x:c>
+      <x:c r="K171" t="str">
+        <x:v>Pass on 2026-07-21: backup /home/ubuntu/deployment-backups/20260721-132209-phase14-clinic-governance-predeploy; backend 4/4; frontend 20/20; four healthy containers; API/frontend/public HTTP 200; /clinics without token HTTP 401.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12902,7 +12949,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de3d0c6712f4ce4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a71dfa0b3ef44c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13276,10 +13323,44 @@
         <x:v>1195</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>R-21</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>/home/ubuntu/deployment-backups/20260721-132209-phase14-clinic-governance-predeploy</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Phase 14 predeployment backup</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Captured the deployment source and MySQL state before applying the clinic-governance migration and rebuilding the affected services.</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Rollback evidence for the targeted de9c7ea deployment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>R-22</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>AWS VM /home/ubuntu/EDR (source marker de9c7ea)</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Phase 14 deployed runtime</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Applied the Phase 14 schema migration and deployed the Database API and frontend payload; mysql and blockchain-api remained healthy and were not rebuilt.</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Live evidence: four healthy containers; database-api, frontend, and public site HTTP 200; protected /clinics returned HTTP 401 without a token.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc225d257014447aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ac7beb05fd423a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14135,10 +14216,32 @@
         <x:v>Phase 14 deployed clinic workflow</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Pending. Migration, Sys Admin bootstrap, login/password replacement, clinic creation, Clinic Admin login, clinic isolation, and activation/deactivation have not yet been executed in the deployment environment.</x:v>
+        <x:v>Pending. Infrastructure and migration deployment passed. Initial Sys Admin bootstrap, forced first-login password replacement, clinic/admin creation, clinic isolation, activation/deactivation, and clinic-bound Fabric wallet enrollment still require authorized runtime execution.</x:v>
       </x:c>
       <x:c r="C77" t="str">
         <x:v>Pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>Phase 14 migration and deployment infrastructure</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>Pass. Corrected migration applied; Organization.IsActive and User.Must_Change_Password exist; Organization_ID and the one-admin-per-clinic primary key were preserved; backend 4/4 and frontend 20/20 passed; all four containers healthy; API/frontend/public HTTP 200.</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>Phase 14 clinic endpoint authentication guard</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>Pass. GET /clinics without a token returned HTTP 401 from the deployed Database API.</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14155,7 +14258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re730c191307c410c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0a35c20f2724b5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14182,7 +14285,7 @@
         <x:v>Initial Sys Admin deployment</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>Source now uses the single-use backend bootstrap:sysadmin command and removes ADMIN_BOOTSTRAP_TOKEN registration. Apply the Phase 14 migration, provide deployment environment credentials, run bootstrap once, and capture first-login forced-password-change evidence.</x:v>
+        <x:v>Migration and application deployment completed 2026-07-21. Provide the authorized email, run the single-use bootstrap:sysadmin command once, and capture forced first-login password-change evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -14202,7 +14305,7 @@
         <x:v>Phase 14 clinic governance deployment</x:v>
       </x:c>
       <x:c r="B5" s="4" t="str">
-        <x:v>Application clinic creation and its single required Clinic Admin are source-complete. Database migration, deployment, authenticated browser/API verification, clinic isolation, and activate/deactivate evidence remain pending.</x:v>
+        <x:v>Migration, Database API, and frontend deployment passed on 2026-07-21. Remaining evidence: initial Sys Admin bootstrap, authenticated clinic/admin creation, clinic isolation, activation/deactivation, and clinic-bound Fabric wallet enrollment.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -14332,7 +14435,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re41453cfc0e6462a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a4cfb1bdf824a83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14987,7 +15090,7 @@
         <x:v>Back up MySQL; apply migration; verify Organization.IsActive, User.Must_Change_Password, unchanged Organization_ID type, and unchanged one-admin-per-clinic Admin primary key.</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>Source corrected after the first deployment attempt exposed the patient foreign-key dependency; migration and deployment remain pending.</x:v>
+        <x:v>Passed 2026-07-21. Backup /home/ubuntu/deployment-backups/20260721-132209-phase14-clinic-governance-predeploy; migration applied; Organization.IsActive and User.Must_Change_Password verified; existing Organization_ID and Admin primary key preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -15007,7 +15110,7 @@
         <x:v>Deploy Database API/frontend, run npm run bootstrap:sysadmin once with environment credentials, change password on first login, create a clinic/admin, enroll its clinic-bound admin wallet identity, and smoke-test role/clinic isolation.</x:v>
       </x:c>
       <x:c r="F33" t="str">
-        <x:v>Source tests/lint/build passed; deployment and live workflow evidence pending.</x:v>
+        <x:v>Partially completed 2026-07-21: commit de9c7ea payload deployed; database-api and web-frontend rebuilt; four containers healthy; HTTP and unauthenticated guard checks passed. Sys Admin bootstrap and authenticated clinic workflow remain pending.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15572,10 +15675,10 @@
         <x:v>FR-01; FR-02; FR-03; SEC-01; SEC-05; multi-clinic onboarding</x:v>
       </x:c>
       <x:c r="F24" t="str">
-        <x:v>Source complete: atomic one-admin clinic creation, system-only lifecycle, inactive-clinic denial, deployment-only Sys Admin bootstrap, forced password replacement, protected UI, 4 backend checks, 20 frontend checks, lint, and build.</x:v>
+        <x:v>Source and deployment infrastructure complete: atomic one-admin clinic creation, system-only lifecycle, inactive-clinic denial, deployment-only Sys Admin bootstrap, forced password replacement, protected UI, migration, focused tests, healthy services, and endpoint/auth-guard checks.</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>Deployment migration and live role/isolation evidence are pending. A new Clinic Admin still requires enrollment of its clinic-bound Fabric wallet identity in the existing Fabric organization; no new blockchain or Fabric organization is created.</x:v>
+        <x:v>Initial Sys Admin bootstrap and authenticated role/isolation workflow evidence remain pending. A new Clinic Admin still requires enrollment of its clinic-bound Fabric wallet identity in the existing Fabric organization; no new blockchain or Fabric organization is created.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15595,7 +15698,7 @@
   <x:sheetData>
     <x:row r="2" ht="21">
       <x:c r="B2" s="86" t="str">
-        <x:v>Remediation Classification Summary — Through Phase 14 Source Completion</x:v>
+        <x:v>Remediation Classification Summary — Through Phase 14 Deployment Infrastructure</x:v>
       </x:c>
       <x:c r="C2" s="86"/>
       <x:c r="D2" s="86"/>
@@ -15640,6 +15743,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="C6" s="20" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$400,B6)</x:f>
         <x:v>60</x:v>
       </x:c>
       <x:c r="D6" s="15" t="s">
@@ -15654,6 +15758,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="C7" s="21" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$400,B7)</x:f>
         <x:v>54</x:v>
       </x:c>
       <x:c r="D7" s="17" t="s">
@@ -15668,6 +15773,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="C8" s="21" t="n">
+        <x:f>COUNTIF('Changes'!$H$2:$H$400,B8)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D8" s="17" t="s">
@@ -15682,7 +15788,8 @@
         <x:v>345</x:v>
       </x:c>
       <x:c r="C9" s="22" t="n">
-        <x:v>37</x:v>
+        <x:f>COUNTIF('Changes'!$H$2:$H$400,B9)</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D9" s="19" t="s">
         <x:v>1695</x:v>
@@ -16008,10 +16115,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F24" s="94" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G24" s="94" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="25">

</xml_diff>